<commit_message>
Rev 2 CAD/drawings/PFD: bolted GFS reactors, contact skid (degasser + lamella), new plant layout, site/diorama, consistency gate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ZeE66f9h61YyPdhTrmHWm
</commit_message>
<xml_diff>
--- a/finance/outputs/BG_Model_Keuangan.xlsx
+++ b/finance/outputs/BG_Model_Keuangan.xlsx
@@ -979,7 +979,7 @@
     <t>Panjang dari model 3D lokasi (site.json)</t>
   </si>
   <si>
-    <t>Lokasi: Efluen AnMBR DN150 HDPE (TK-301 -&gt; kolam fakultatif)</t>
+    <t>Lokasi: Efluen settler DN150 HDPE (TK-301 -&gt; kolam fakultatif)</t>
   </si>
   <si>
     <t>Lokasi: Bypass darurat DN150 (TK-101 -&gt; kolam pendingin)</t>
@@ -1654,7 +1654,7 @@
     <t>POME 85 °C DN150 (fat pit -&gt; PM-1)</t>
   </si>
   <si>
-    <t>Efluen AnMBR DN150 HDPE (TK-301 -&gt; kolam fakultatif)</t>
+    <t>Efluen settler DN150 HDPE (TK-301 -&gt; kolam fakultatif)</t>
   </si>
   <si>
     <t>Bypass darurat DN150 (TK-101 -&gt; kolam pendingin)</t>
@@ -2542,7 +2542,7 @@
     <t>3.3 (FCI/kWe terpasang)</t>
   </si>
   <si>
-    <t>0.24</t>
+    <t>0.38</t>
   </si>
   <si>
     <t>10</t>
@@ -2599,7 +2599,7 @@
     <t>3 Aset dapat dipindah</t>
   </si>
   <si>
-    <t>Bila PKS tutup th 8: NPV pengembang 220,392 vs tangki tetap -824,836 (USD)</t>
+    <t>Bila PKS tutup th 8: NPV pengembang 198,908 vs tangki tetap -837,849 (USD)</t>
   </si>
   <si>
     <t>Model skenario relokasi</t>
@@ -2611,7 +2611,7 @@
     <t>4 Lahan &amp; bau</t>
   </si>
   <si>
-    <t>Membebaskan 1,1 ha kolam anaerobik; plot 0.24 ha; reaktor tertutup</t>
+    <t>Membebaskan 1,1 ha kolam anaerobik; plot 0.38 ha; reaktor tertutup</t>
   </si>
   <si>
     <t>Model 3D lokasi</t>
@@ -5281,7 +5281,7 @@
     <t>Jendela fee (min - maks USD/t TBS)</t>
   </si>
   <si>
-    <t>0.58 - 1.90</t>
+    <t>0.60 - 1.90</t>
   </si>
 </sst>
 </file>
@@ -5556,67 +5556,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>-4546175.134666292</c:v>
+                  <c:v>-4545840.428041292</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-4248478.403445761</c:v>
+                  <c:v>-4250713.779160254</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-3164022.8413079483</c:v>
+                  <c:v>-3169143.026761141</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2449418.029367366</c:v>
+                  <c:v>-2457446.8882465325</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1723982.8274934893</c:v>
+                  <c:v>-1734978.5332671492</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-992976.8553327934</c:v>
+                  <c:v>-1006998.7449388367</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-256288.697479542</c:v>
+                  <c:v>-273397.29459461605</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>486195.28978011606</c:v>
+                  <c:v>465938.2510058305</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>992576.9009874985</c:v>
+                  <c:v>974308.1800427171</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1586584.7435387785</c:v>
+                  <c:v>1565762.1876677717</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2185382.840451277</c:v>
+                  <c:v>2161955.3729555206</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2694515.1645594793</c:v>
+                  <c:v>2668430.687206478</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3032842.4729034537</c:v>
+                  <c:v>3004047.8454960627</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3456870.098093314</c:v>
+                  <c:v>3425311.1176304454</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3886329.3447283865</c:v>
+                  <c:v>3851950.7241489305</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4321328.845237575</c:v>
+                  <c:v>4284074.1917392</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4510951.436054047</c:v>
+                  <c:v>4470763.228978375</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4958381.562455786</c:v>
+                  <c:v>4915201.130731271</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5411691.050590768</c:v>
+                  <c:v>5365458.549724433</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>5870997.487693658</c:v>
+                  <c:v>5821651.876302666</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>6469309.43000992</c:v>
+                  <c:v>6416453.151137525</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5717,67 +5717,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>-4546175.134666292</c:v>
+                  <c:v>-4545840.428041292</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-4274910.435711879</c:v>
+                  <c:v>-4276917.617791039</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-3374479.951776244</c:v>
+                  <c:v>-3378882.4100841125</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-2833820.7738280753</c:v>
+                  <c:v>-2840423.8903978663</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-2333699.321225392</c:v>
+                  <c:v>-2342347.8083185474</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-1874483.3358658473</c:v>
+                  <c:v>-1885032.8635022957</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-1452787.8271118829</c:v>
+                  <c:v>-1465104.2498443357</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1065510.9271014105</c:v>
+                  <c:v>-1079469.5653517272</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-824835.5604149617</c:v>
+                  <c:v>-837849.1818792933</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-567579.7993422421</c:v>
+                  <c:v>-581699.4478663823</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-331274.9923629672</c:v>
+                  <c:v>-346422.6220077197</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-148194.51758101842</c:v>
+                  <c:v>-164297.58965818133</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-37336.367422023264</c:v>
+                  <c:v>-54327.461879506416</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>89266.61596159647</c:v>
+                  <c:v>71450.16173234754</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>206106.45788176844</c:v>
+                  <c:v>187522.88475107512</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>313945.7368806239</c:v>
+                  <c:v>294649.1759970937</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>356780.6122686951</c:v>
+                  <c:v>336821.3750585379</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>448878.9663709626</c:v>
+                  <c:v>428303.8140737304</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>533902.797475987</c:v>
+                  <c:v>512755.19166073424</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>612402.42702482</c:v>
+                  <c:v>590722.7624287857</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>705580.1216725708</c:v>
+                  <c:v>683353.7257154249</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6706,127 +6706,127 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="41"/>
                 <c:pt idx="0">
-                  <c:v>3269267.1996731823</c:v>
+                  <c:v>3233928.145940558</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2972567.0333865928</c:v>
+                  <c:v>2938797.2024187334</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2693302.568581547</c:v>
+                  <c:v>2660999.066889058</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2430195.517452772</c:v>
+                  <c:v>2399263.4820770836</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2182074.8672046014</c:v>
+                  <c:v>2152426.7692785813</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1947866.9894888161</c:v>
+                  <c:v>1919422.003034134</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1726586.7297566542</c:v>
+                  <c:v>1699270.159213186</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1517329.3735594128</c:v>
+                  <c:v>1491072.1342262463</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1319263.3982093295</c:v>
+                  <c:v>1294001.5443856898</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1131623.9282763898</c:v>
+                  <c:v>1107298.2244328542</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>953706.8223032231</c:v>
+                  <c:v>930262.3530964057</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>784863.3260097193</c:v>
+                  <c:v>762249.1413840966</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>624495.2342506241</c:v>
+                  <c:v>602664.0262551631</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>472050.51019139664</c:v>
+                  <c:v>450958.3184813967</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>327019.3156711395</c:v>
+                  <c:v>306625.2589719249</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>188930.41161014634</c:v>
+                  <c:v>169196.4426928563</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>57347.89166374598</c:v>
+                  <c:v>38238.573628280894</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-68131.78381224057</c:v>
+                  <c:v>-86649.4819330393</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-187882.48298077402</c:v>
+                  <c:v>-205839.37308546156</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-302250.8533621847</c:v>
+                  <c:v>-319675.6992275151</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-411558.55199828476</c:v>
+                  <c:v>-428478.2257648624</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-516104.27621552773</c:v>
+                  <c:v>-532543.9017272156</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-616165.6140897981</c:v>
+                  <c:v>-632148.6982749056</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-712000.7317777171</c:v>
+                  <c:v>-727549.2851458985</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-803849.9131475608</c:v>
+                  <c:v>-818984.560373871</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-891936.965595297</c:v>
+                  <c:v>-906677.0470706664</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-976470.5045463681</c:v>
+                  <c:v>-990834.1696907661</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-1057645.1279046785</c:v>
+                  <c:v>-1071649.4209645549</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-1135642.490599939</c:v>
+                  <c:v>-1149303.4295841798</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-1210632.2883898343</c:v>
+                  <c:v>-1223964.9377378388</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-1282773.1591811022</c:v>
+                  <c:v>-1295791.6967017895</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-1352213.509333176</c:v>
+                  <c:v>-1364931.2879043529</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-1419092.271689017</c:v>
+                  <c:v>-1431521.8761619083</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-1483539.6014320944</c:v>
+                  <c:v>-1495692.9011455283</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-1545677.515287707</c:v>
+                  <c:v>-1557565.7125599594</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-1605620.4790647118</c:v>
+                  <c:v>-1617254.153998071</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-1663475.948063523</c:v>
+                  <c:v>-1674865.0999667633</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-1719344.864452985</c:v>
+                  <c:v>-1730498.950159903</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-1773322.1153371783</c:v>
+                  <c:v>-1784250.0846748513</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-1825496.9548892095</c:v>
+                  <c:v>-1836207.2835274225</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-1875953.39361871</c:v>
+                  <c:v>-1886454.113511846</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6917,94 +6917,94 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
                 <c:pt idx="0">
-                  <c:v>-2206213.721122548</c:v>
+                  <c:v>-2232479.874163236</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-2041185.286519913</c:v>
+                  <c:v>-2067363.791636461</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-1876156.85191728</c:v>
+                  <c:v>-1902247.709109687</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-1711128.417314646</c:v>
+                  <c:v>-1737131.626582914</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1546099.982712012</c:v>
+                  <c:v>-1572015.54405614</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-1381071.548109378</c:v>
+                  <c:v>-1406899.461529366</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-1216043.113506744</c:v>
+                  <c:v>-1241783.379002592</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-1051014.67890411</c:v>
+                  <c:v>-1076667.296475818</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-885986.2443014761</c:v>
+                  <c:v>-911551.2139490441</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-720957.8096988421</c:v>
+                  <c:v>-746435.1314222702</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-555929.3750962083</c:v>
+                  <c:v>-581319.0488954963</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-390900.9404935744</c:v>
+                  <c:v>-416202.9663687225</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-225872.5058909403</c:v>
+                  <c:v>-251086.8838419486</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-60844.0712883065</c:v>
+                  <c:v>-85970.80131517467</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>104184.3633143273</c:v>
+                  <c:v>79145.28121159924</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>269212.7979169614</c:v>
+                  <c:v>244261.3637383732</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>434241.2325195954</c:v>
+                  <c:v>409377.4462651468</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>599269.6671222295</c:v>
+                  <c:v>574493.5287919207</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>764298.1017248633</c:v>
+                  <c:v>739609.6113186947</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>929326.5363274971</c:v>
+                  <c:v>904725.6938454686</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>1094354.970930131</c:v>
+                  <c:v>1069841.776372242</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1259383.405532765</c:v>
+                  <c:v>1234957.858899016</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1424411.840135399</c:v>
+                  <c:v>1400073.94142579</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1589440.274738033</c:v>
+                  <c:v>1565190.023952564</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1754468.709340667</c:v>
+                  <c:v>1730306.106479338</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1919497.143943301</c:v>
+                  <c:v>1895422.189006112</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>2084525.578545935</c:v>
+                  <c:v>2060538.271532886</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>2249554.013148569</c:v>
+                  <c:v>2225654.354059659</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>2414582.447751202</c:v>
+                  <c:v>2390770.436586434</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>2579610.882353836</c:v>
+                  <c:v>2555886.519113207</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7016,10 +7016,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="30"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -7031,28 +7031,28 @@
                   <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>32</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>47</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>75</c:v>
+                  <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>107</c:v>
+                  <c:v>105</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>116</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>155</c:v>
+                  <c:v>158</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>191</c:v>
+                  <c:v>190</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>211</c:v>
+                  <c:v>207</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>236</c:v>
@@ -7061,34 +7061,34 @@
                   <c:v>283</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>242</c:v>
+                  <c:v>243</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>269</c:v>
+                  <c:v>272</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>254</c:v>
+                  <c:v>250</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>177</c:v>
+                  <c:v>181</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>168</c:v>
+                  <c:v>167</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>136</c:v>
+                  <c:v>135</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>102</c:v>
+                  <c:v>104</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>67</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>44</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>24</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="25">
                   <c:v>10</c:v>
@@ -8436,7 +8436,7 @@
       </c>
       <c r="B4" s="3">
         <f>FCI</f>
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B5" s="3">
         <f>FCI26/t_P_gross</f>
-        <v>3564.1810183390016</v>
+        <v>3563.918609838625</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B7" s="3">
         <f>'Arus Kas'!F20</f>
-        <v>721426.3945163141</v>
+        <v>718513.0258951411</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="B8" s="3">
         <f>Indikator!B4</f>
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="B9" s="4">
         <f>Indikator!B5</f>
-        <v>0.12225595720238847</v>
+        <v>0.12150604052544578</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="B10" s="4">
         <f>Indikator!B6</f>
-        <v>0.14128956808421878</v>
+        <v>0.14006099840090447</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="B12" s="5">
         <f>Indikator!B8</f>
-        <v>6.345177407024556</v>
+        <v>6.369787840205327</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="B13" s="5">
         <f>Indikator!B9</f>
-        <v>12.294909064732625</v>
+        <v>12.431932646836765</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="B14" s="5">
         <f>Indikator!B11</f>
-        <v>1.3180782341273873</v>
+        <v>1.3056039524321026</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B16" s="5">
         <f>Indikator!B17</f>
-        <v>0.5828638963044959</v>
+        <v>0.5961118395426859</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="B17" s="4">
         <f>'Monte Carlo'!B9</f>
-        <v>0.609</v>
+        <v>0.5943333333333334</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -8562,7 +8562,7 @@
       </c>
       <c r="B18" s="3">
         <f>Armada!B60</f>
-        <v>1103176.7165093392</v>
+        <v>880902.5235970457</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B19" s="4">
         <f>Armada!B61</f>
-        <v>0.10144038785123799</v>
+        <v>0.10064111031235168</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -9468,85 +9468,85 @@
         <v>0</v>
       </c>
       <c r="D12" s="12">
-        <v>347998.7762134077</v>
+        <v>350798.7076120677</v>
       </c>
       <c r="E12" s="12">
-        <v>695707.6828106854</v>
+        <v>701419.9506994513</v>
       </c>
       <c r="F12" s="12">
-        <v>1391559.054240951</v>
+        <v>1403212.634765911</v>
       </c>
       <c r="G12" s="12">
-        <v>2115922.758993776</v>
+        <v>2133753.129063067</v>
       </c>
       <c r="H12" s="12">
-        <v>2865129.788098795</v>
+        <v>2889379.429397822</v>
       </c>
       <c r="I12" s="12">
-        <v>3640801.689318296</v>
+        <v>3671720.293721602</v>
       </c>
       <c r="J12" s="12">
-        <v>4444237.306995427</v>
+        <v>4482081.97553878</v>
       </c>
       <c r="K12" s="12">
-        <v>5640806.857060552</v>
+        <v>5689059.252160678</v>
       </c>
       <c r="L12" s="12">
-        <v>5774883.299842918</v>
+        <v>5824100.742845046</v>
       </c>
       <c r="M12" s="12">
-        <v>5890380.965839776</v>
+        <v>5940582.757701947</v>
       </c>
       <c r="N12" s="12">
-        <v>6008188.585156572</v>
+        <v>6059394.412855987</v>
       </c>
       <c r="O12" s="12">
-        <v>6112829.077294258</v>
+        <v>6165059.021547661</v>
       </c>
       <c r="P12" s="12">
-        <v>6219251.913683388</v>
+        <v>6272526.456821859</v>
       </c>
       <c r="Q12" s="12">
-        <v>6311336.111837278</v>
+        <v>6365676.145838519</v>
       </c>
       <c r="R12" s="12">
-        <v>6404615.977151849</v>
+        <v>6460042.811833113</v>
       </c>
       <c r="S12" s="12">
-        <v>6499102.502634268</v>
+        <v>6555637.874009158</v>
       </c>
       <c r="T12" s="12">
-        <v>6594806.642745123</v>
+        <v>6652472.72154751</v>
       </c>
       <c r="U12" s="12">
-        <v>6691739.307459358</v>
+        <v>6750558.707837793</v>
       </c>
       <c r="V12" s="12">
-        <v>6772079.987353325</v>
+        <v>6832075.77573933</v>
       </c>
       <c r="W12" s="12">
-        <v>6907521.587100391</v>
+        <v>6968717.291254115</v>
       </c>
       <c r="X12" s="12">
-        <v>6538128.16351398</v>
+        <v>6596387.230980024</v>
       </c>
       <c r="Y12" s="12">
-        <v>6181478.531144211</v>
+        <v>6236658.412151303</v>
       </c>
       <c r="Z12" s="12">
-        <v>5321036.922185847</v>
+        <v>5368661.685364524</v>
       </c>
       <c r="AA12" s="12">
-        <v>4431821.514738013</v>
+        <v>4471566.720994055</v>
       </c>
       <c r="AB12" s="12">
-        <v>3510220.744106348</v>
+        <v>3541752.054959084</v>
       </c>
       <c r="AC12" s="12">
-        <v>2553931.435632474</v>
+        <v>2576904.318170418</v>
       </c>
       <c r="AD12" s="12">
-        <v>1561132.377160026</v>
+        <v>1575191.818769455</v>
       </c>
     </row>
     <row r="13" spans="1:30">
@@ -9560,85 +9560,85 @@
         <v>0</v>
       </c>
       <c r="D13" s="12">
-        <v>373608.71780944</v>
+        <v>370808.78641078</v>
       </c>
       <c r="E13" s="12">
-        <v>1064434.358363569</v>
+        <v>1058722.090474803</v>
       </c>
       <c r="F13" s="12">
-        <v>2205756.97606667</v>
+        <v>2194103.39554171</v>
       </c>
       <c r="G13" s="12">
-        <v>3666641.803865083</v>
+        <v>3648811.433795792</v>
       </c>
       <c r="H13" s="12">
-        <v>5187403.263305882</v>
+        <v>5163153.622006856</v>
       </c>
       <c r="I13" s="12">
-        <v>6735312.031506472</v>
+        <v>6704393.427103165</v>
       </c>
       <c r="J13" s="12">
-        <v>8310663.281313278</v>
+        <v>8272818.612769923</v>
       </c>
       <c r="K13" s="12">
-        <v>10343441.33814973</v>
+        <v>10295188.94304961</v>
       </c>
       <c r="L13" s="12">
-        <v>11420294.76778579</v>
+        <v>11371077.32478365</v>
       </c>
       <c r="M13" s="12">
-        <v>11614572.80775545</v>
+        <v>11564371.01589328</v>
       </c>
       <c r="N13" s="12">
-        <v>11559206.38906034</v>
+        <v>11508000.56136093</v>
       </c>
       <c r="O13" s="12">
-        <v>11412459.34285688</v>
+        <v>11360229.39860348</v>
       </c>
       <c r="P13" s="12">
-        <v>11114748.09722355</v>
+        <v>11061473.55408508</v>
       </c>
       <c r="Q13" s="12">
-        <v>10727002.28743392</v>
+        <v>10672662.25343268</v>
       </c>
       <c r="R13" s="12">
-        <v>10342645.86723738</v>
+        <v>10287219.03255612</v>
       </c>
       <c r="S13" s="12">
-        <v>9961759.544761833</v>
+        <v>9905224.173386943</v>
       </c>
       <c r="T13" s="12">
-        <v>9584425.900704468</v>
+        <v>9526759.821902078</v>
       </c>
       <c r="U13" s="12">
-        <v>9057140.562360931</v>
+        <v>8998321.161982495</v>
       </c>
       <c r="V13" s="12">
-        <v>8903308.471422685</v>
+        <v>8843312.683036681</v>
       </c>
       <c r="W13" s="12">
-        <v>9026042.801989879</v>
+        <v>8964847.097836154</v>
       </c>
       <c r="X13" s="12">
-        <v>8578982.085296113</v>
+        <v>8520723.01783007</v>
       </c>
       <c r="Y13" s="12">
-        <v>8088630.201310921</v>
+        <v>8033450.320303828</v>
       </c>
       <c r="Z13" s="12">
-        <v>6954587.932763071</v>
+        <v>6906963.169584394</v>
       </c>
       <c r="AA13" s="12">
-        <v>5779546.306348057</v>
+        <v>5739801.100092012</v>
       </c>
       <c r="AB13" s="12">
-        <v>4564976.202486677</v>
+        <v>4533444.891633941</v>
       </c>
       <c r="AC13" s="12">
-        <v>3310982.393455358</v>
+        <v>3288009.510917413</v>
       </c>
       <c r="AD13" s="12">
-        <v>2017128.518469475</v>
+        <v>2003069.076860046</v>
       </c>
     </row>
     <row r="14" spans="1:30">
@@ -9649,28 +9649,28 @@
         <v>0</v>
       </c>
       <c r="C14" s="12">
-        <v>4914783.929368964</v>
+        <v>4914422.084368965</v>
       </c>
       <c r="D14" s="12">
-        <v>3926912.359565803</v>
+        <v>3926623.245410803</v>
       </c>
       <c r="E14" s="12">
-        <v>7643267.286254702</v>
+        <v>7642704.559980071</v>
       </c>
       <c r="F14" s="12">
-        <v>7505013.359785681</v>
+        <v>7504460.812288538</v>
       </c>
       <c r="G14" s="12">
-        <v>7464595.91283268</v>
+        <v>7464046.341021</v>
       </c>
       <c r="H14" s="12">
-        <v>7472273.903288389</v>
+        <v>7471723.766193982</v>
       </c>
       <c r="I14" s="12">
-        <v>7508882.563074235</v>
+        <v>7508329.730711697</v>
       </c>
       <c r="J14" s="12">
-        <v>11317219.9450405</v>
+        <v>11316386.72846173</v>
       </c>
       <c r="K14" s="12">
         <v>215116.662352016</v>
@@ -9833,88 +9833,88 @@
         <v>-1050000</v>
       </c>
       <c r="C16" s="13">
-        <v>-5950410.16159955</v>
+        <v>-5950008.513649551</v>
       </c>
       <c r="D16" s="13">
-        <v>-4619781.772144131</v>
+        <v>-4622030.655482906</v>
       </c>
       <c r="E16" s="13">
-        <v>-7620055.290658608</v>
+        <v>-7624943.365210059</v>
       </c>
       <c r="F16" s="13">
-        <v>-6596500.434031126</v>
+        <v>-6607084.162325319</v>
       </c>
       <c r="G16" s="13">
-        <v>-4802711.951892517</v>
+        <v>-4819486.515808642</v>
       </c>
       <c r="H16" s="13">
-        <v>-3390038.5948078</v>
+        <v>-3413210.75282277</v>
       </c>
       <c r="I16" s="13">
-        <v>-1973569.369405623</v>
+        <v>-2003386.648832022</v>
       </c>
       <c r="J16" s="13">
-        <v>-4738202.750028003</v>
+        <v>-4768680.729286296</v>
       </c>
       <c r="K16" s="13">
-        <v>9395498.43702027</v>
+        <v>9366765.654914886</v>
       </c>
       <c r="L16" s="13">
-        <v>10946179.01299079</v>
+        <v>10907456.21883777</v>
       </c>
       <c r="M16" s="13">
-        <v>9469856.897373257</v>
+        <v>9438560.577877358</v>
       </c>
       <c r="N16" s="13">
-        <v>8998577.333122246</v>
+        <v>8965012.358175676</v>
       </c>
       <c r="O16" s="13">
-        <v>8485107.45700587</v>
+        <v>8444367.02897222</v>
       </c>
       <c r="P16" s="13">
-        <v>7973791.759880687</v>
+        <v>7932259.785294156</v>
       </c>
       <c r="Q16" s="13">
-        <v>7245892.634232231</v>
+        <v>7203555.951164538</v>
       </c>
       <c r="R16" s="13">
-        <v>6477047.596652895</v>
+        <v>6433880.52830594</v>
       </c>
       <c r="S16" s="13">
-        <v>6329923.694298236</v>
+        <v>6285917.217230777</v>
       </c>
       <c r="T16" s="13">
-        <v>6009549.007525063</v>
+        <v>5964662.400916256</v>
       </c>
       <c r="U16" s="13">
-        <v>5335767.792142667</v>
+        <v>5289983.453401683</v>
       </c>
       <c r="V16" s="13">
-        <v>5016809.41809607</v>
+        <v>4970109.392580268</v>
       </c>
       <c r="W16" s="13">
-        <v>5494969.180297857</v>
+        <v>5446999.896353061</v>
       </c>
       <c r="X16" s="13">
-        <v>5108932.039249229</v>
+        <v>5063241.845234989</v>
       </c>
       <c r="Y16" s="13">
-        <v>4824463.921219246</v>
+        <v>4780814.821299756</v>
       </c>
       <c r="Z16" s="13">
-        <v>3605413.999982409</v>
+        <v>3567631.748609357</v>
       </c>
       <c r="AA16" s="13">
-        <v>3519446.620084026</v>
+        <v>3487783.482056582</v>
       </c>
       <c r="AB16" s="13">
-        <v>2533320.196790751</v>
+        <v>2508036.134654803</v>
       </c>
       <c r="AC16" s="13">
-        <v>1515702.151339838</v>
+        <v>1497065.056310079</v>
       </c>
       <c r="AD16" s="13">
-        <v>616539.373612687</v>
+        <v>604440.0968600379</v>
       </c>
     </row>
     <row r="17" spans="1:30">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="B19" s="3">
         <f>B16+NPV(WACC,C16:AD16)</f>
-        <v>1103176.7165093392</v>
+        <v>880902.5235970457</v>
       </c>
     </row>
     <row r="20" spans="1:30">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B20" s="4">
         <f>IRR(B16:AD16)</f>
-        <v>0.10144038785123799</v>
+        <v>0.10064111031235168</v>
       </c>
     </row>
     <row r="21" spans="1:30">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="B21" s="3">
         <f>-MIN(B17:AD17)</f>
-        <v>40741270.32456736</v>
+        <v>40858831.34341757</v>
       </c>
     </row>
     <row r="23" spans="1:30">
@@ -10096,13 +10096,13 @@
         <v>1.2</v>
       </c>
       <c r="D24" s="12">
-        <v>4914783.929368964</v>
+        <v>4914422.084368965</v>
       </c>
       <c r="E24" s="13">
-        <v>-153781.6032148016</v>
+        <v>-176398.1055447065</v>
       </c>
       <c r="F24" s="15">
-        <v>0.09277729210484797</v>
+        <v>0.09208460725740375</v>
       </c>
     </row>
     <row r="25" spans="1:30">
@@ -10116,13 +10116,13 @@
         <v>0.9400000000000001</v>
       </c>
       <c r="D25" s="12">
-        <v>3926912.359565803</v>
+        <v>3926623.245410803</v>
       </c>
       <c r="E25" s="13">
-        <v>927335.8088371551</v>
+        <v>904860.7149566974</v>
       </c>
       <c r="F25" s="15">
-        <v>0.1310593617002231</v>
+        <v>0.1302892255551777</v>
       </c>
     </row>
     <row r="26" spans="1:30">
@@ -10136,13 +10136,13 @@
         <v>0.907723591787405</v>
       </c>
       <c r="D26" s="12">
-        <v>3867917.03350278</v>
+        <v>3867632.262807038</v>
       </c>
       <c r="E26" s="13">
-        <v>1036803.747391219</v>
+        <v>1014072.050608469</v>
       </c>
       <c r="F26" s="15">
-        <v>0.1353528122725018</v>
+        <v>0.1345741659514377</v>
       </c>
     </row>
     <row r="27" spans="1:30">
@@ -10156,13 +10156,13 @@
         <v>0.886</v>
       </c>
       <c r="D27" s="12">
-        <v>3775350.252751923</v>
+        <v>3775072.297173033</v>
       </c>
       <c r="E27" s="13">
-        <v>1129281.804864095</v>
+        <v>1106727.017796097</v>
       </c>
       <c r="F27" s="15">
-        <v>0.1395163057006032</v>
+        <v>0.1387365913969127</v>
       </c>
     </row>
     <row r="28" spans="1:30">
@@ -10176,13 +10176,13 @@
         <v>0.8697920330082306</v>
       </c>
       <c r="D28" s="12">
-        <v>3780411.922226204</v>
+        <v>3780133.593988044</v>
       </c>
       <c r="E28" s="13">
-        <v>1174227.229697527</v>
+        <v>1151216.756519271</v>
       </c>
       <c r="F28" s="15">
-        <v>0.1409898983363913</v>
+        <v>0.1401994361909087</v>
       </c>
     </row>
     <row r="29" spans="1:30">
@@ -10196,13 +10196,13 @@
         <v>0.8569512326086645</v>
       </c>
       <c r="D29" s="12">
-        <v>3724601.437559477</v>
+        <v>3724327.218300494</v>
       </c>
       <c r="E29" s="13">
-        <v>1229358.318528496</v>
+        <v>1206506.529402385</v>
       </c>
       <c r="F29" s="15">
-        <v>0.1435532368109953</v>
+        <v>0.1427654555591993</v>
       </c>
     </row>
     <row r="30" spans="1:30">
@@ -10216,13 +10216,13 @@
         <v>0.8463687003893453</v>
       </c>
       <c r="D30" s="12">
-        <v>3752178.277345886</v>
+        <v>3751902.027775553</v>
       </c>
       <c r="E30" s="13">
-        <v>1252823.551988613</v>
+        <v>1229511.704081826</v>
       </c>
       <c r="F30" s="15">
-        <v>0.1439983148890152</v>
+        <v>0.1432023490833507</v>
       </c>
     </row>
     <row r="31" spans="1:30">
@@ -10236,13 +10236,13 @@
         <v>0.8374</v>
       </c>
       <c r="D31" s="12">
-        <v>3712417.635486795</v>
+        <v>3712144.313245447</v>
       </c>
       <c r="E31" s="13">
-        <v>1291962.55522449</v>
+        <v>1268648.14532553</v>
       </c>
       <c r="F31" s="15">
-        <v>0.1458413336941489</v>
+        <v>0.1450408549925053</v>
       </c>
     </row>
     <row r="32" spans="1:30">
@@ -10256,13 +10256,13 @@
         <v>0.8296387427625059</v>
       </c>
       <c r="D32" s="12">
-        <v>3751570.109516255</v>
+        <v>3751293.90472154</v>
       </c>
       <c r="E32" s="13">
-        <v>1305045.352398708</v>
+        <v>1281262.392885397</v>
       </c>
       <c r="F32" s="15">
-        <v>0.1457638144951903</v>
+        <v>0.1449563751352272</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -10276,13 +10276,13 @@
         <v>0.8228128297074077</v>
       </c>
       <c r="D33" s="12">
-        <v>3720703.793772133</v>
+        <v>3720429.861472442</v>
       </c>
       <c r="E33" s="13">
-        <v>1335429.088055444</v>
+        <v>1311644.139659267</v>
       </c>
       <c r="F33" s="15">
-        <v>0.1471992076932924</v>
+        <v>0.1463881847897248</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -10296,13 +10296,13 @@
         <v>0.8167315110307659</v>
       </c>
       <c r="D34" s="12">
-        <v>3767068.572957645</v>
+        <v>3766791.227107375</v>
       </c>
       <c r="E34" s="13">
-        <v>1342444.803835907</v>
+        <v>1318182.349104643</v>
       </c>
       <c r="F34" s="15">
-        <v>0.1468079469752275</v>
+        <v>0.1459907372781406</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -10316,13 +10316,13 @@
         <v>0.8112561093477982</v>
       </c>
       <c r="D35" s="12">
-        <v>3741813.99011659</v>
+        <v>3741538.503604321</v>
       </c>
       <c r="E35" s="13">
-        <v>1367304.543350167</v>
+        <v>1343040.461330194</v>
       </c>
       <c r="F35" s="15">
-        <v>0.1479790906672458</v>
+        <v>0.1471589092958512</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -10336,13 +10336,13 @@
         <v>0.8062827794850708</v>
       </c>
       <c r="D36" s="12">
-        <v>3793252.651652312</v>
+        <v>3792973.378031037</v>
       </c>
       <c r="E36" s="13">
-        <v>1370378.81658107</v>
+        <v>1345627.945286212</v>
       </c>
       <c r="F36" s="15">
-        <v>0.147382649491598</v>
+        <v>0.1465568183947306</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -10356,13 +10356,13 @@
         <v>0.8017318303504107</v>
       </c>
       <c r="D37" s="12">
-        <v>3771842.173453077</v>
+        <v>3771564.476152266</v>
       </c>
       <c r="E37" s="13">
-        <v>1391454.552191457</v>
+        <v>1366702.301304243</v>
       </c>
       <c r="F37" s="15">
-        <v>0.1483687788039902</v>
+        <v>0.1475404098189943</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -10376,13 +10376,13 @@
         <v>0.7975408306534101</v>
       </c>
       <c r="D38" s="12">
-        <v>3752125.119935111</v>
+        <v>3751848.874278428</v>
       </c>
       <c r="E38" s="13">
-        <v>1410863.339005728</v>
+        <v>1386109.817642626</v>
       </c>
       <c r="F38" s="15">
-        <v>0.1492848325037082</v>
+        <v>0.1484540960365102</v>
       </c>
     </row>
   </sheetData>
@@ -10423,13 +10423,13 @@
         <v>496</v>
       </c>
       <c r="B4" s="12">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C4" s="10">
         <v>140</v>
       </c>
       <c r="D4" s="12">
-        <v>22740.2</v>
+        <v>22565.2</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -10437,13 +10437,13 @@
         <v>497</v>
       </c>
       <c r="B5" s="12">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C5" s="10">
         <v>70</v>
       </c>
       <c r="D5" s="12">
-        <v>10345.5</v>
+        <v>10755</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -10451,13 +10451,13 @@
         <v>498</v>
       </c>
       <c r="B6" s="12">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C6" s="10">
         <v>70</v>
       </c>
       <c r="D6" s="12">
-        <v>5139.750000000001</v>
+        <v>4492.250000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -10465,13 +10465,13 @@
         <v>499</v>
       </c>
       <c r="B7" s="12">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C7" s="10">
         <v>45</v>
       </c>
       <c r="D7" s="12">
-        <v>4151.25</v>
+        <v>3937.5</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -10479,13 +10479,13 @@
         <v>500</v>
       </c>
       <c r="B8" s="12">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="C8" s="10">
         <v>40</v>
       </c>
       <c r="D8" s="12">
-        <v>27874</v>
+        <v>28232</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -10517,7 +10517,7 @@
         <v>504</v>
       </c>
       <c r="B14" s="12">
-        <v>2410.3148</v>
+        <v>3756.805</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -10544,7 +10544,7 @@
         <v>509</v>
       </c>
       <c r="B19" s="10">
-        <v>16.1</v>
+        <v>15.8</v>
       </c>
       <c r="C19" s="12">
         <v>15</v>
@@ -10558,7 +10558,7 @@
         <v>511</v>
       </c>
       <c r="B20" s="10">
-        <v>30.5</v>
+        <v>20.8</v>
       </c>
       <c r="C20" s="12">
         <v>15</v>
@@ -10572,7 +10572,7 @@
         <v>512</v>
       </c>
       <c r="B21" s="10">
-        <v>142.9</v>
+        <v>141.5</v>
       </c>
       <c r="C21" s="12">
         <v>30</v>
@@ -10586,7 +10586,7 @@
         <v>513</v>
       </c>
       <c r="B22" s="10">
-        <v>208.7</v>
+        <v>208</v>
       </c>
       <c r="C22" s="12">
         <v>30</v>
@@ -10600,7 +10600,7 @@
         <v>514</v>
       </c>
       <c r="B23" s="10">
-        <v>17.2</v>
+        <v>21.5</v>
       </c>
       <c r="C23" s="12">
         <v>10</v>
@@ -10614,7 +10614,7 @@
         <v>515</v>
       </c>
       <c r="B24" s="10">
-        <v>20.6</v>
+        <v>20.9</v>
       </c>
       <c r="C24" s="12">
         <v>20</v>
@@ -10628,7 +10628,7 @@
         <v>516</v>
       </c>
       <c r="B25" s="10">
-        <v>138.2</v>
+        <v>137.1</v>
       </c>
       <c r="C25" s="12">
         <v>30</v>
@@ -12042,7 +12042,7 @@
       </c>
       <c r="E65" s="3">
         <f>Indikator!B4</f>
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="E66" s="4">
         <f>Indikator!B5</f>
-        <v>0.12225595720238847</v>
+        <v>0.12150604052544578</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -12073,7 +12073,7 @@
         <v>706</v>
       </c>
       <c r="B70" s="5">
-        <v>0.5828638963044959</v>
+        <v>0.5961118395426859</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -12089,7 +12089,7 @@
         <v>708</v>
       </c>
       <c r="B72" s="5">
-        <v>1.322026350809778</v>
+        <v>1.308778407571588</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -12263,7 +12263,7 @@
         <v>0.53</v>
       </c>
       <c r="D4" s="10">
-        <v>1.45731278089607</v>
+        <v>1.470562272108429</v>
       </c>
       <c r="E4" s="10">
         <v>0.5954357385339313</v>
@@ -12273,10 +12273,10 @@
         <v>Tidak</v>
       </c>
       <c r="G4" s="13">
-        <v>-781824.2484732983</v>
+        <v>-804731.0521045423</v>
       </c>
       <c r="H4" s="15">
-        <v>0.06387322919803462</v>
+        <v>0.06279156195873759</v>
       </c>
       <c r="I4" s="15">
         <v>-0.324296950400979</v>
@@ -12296,7 +12296,7 @@
         <v>0.53</v>
       </c>
       <c r="D5" s="10">
-        <v>1.075533801602242</v>
+        <v>1.087224529142558</v>
       </c>
       <c r="E5" s="10">
         <v>0.5806279023112015</v>
@@ -12306,10 +12306,10 @@
         <v>Tidak</v>
       </c>
       <c r="G5" s="13">
-        <v>-145022.4857663354</v>
+        <v>-167468.3091242231</v>
       </c>
       <c r="H5" s="15">
-        <v>0.09145611344978</v>
+        <v>0.09051358116000063</v>
       </c>
       <c r="I5" s="15">
         <v>-0.3421325137388238</v>
@@ -12329,7 +12329,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="10">
-        <v>0.5828638963044959</v>
+        <v>0.5961118395426859</v>
       </c>
       <c r="E6" s="10">
         <v>1.904890247114274</v>
@@ -12339,10 +12339,10 @@
         <v>Ya</v>
       </c>
       <c r="G6" s="13">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
       <c r="H6" s="15">
-        <v>0.1222559572023885</v>
+        <v>0.1215060405254458</v>
       </c>
       <c r="I6" s="15">
         <v>0.2103322723258169</v>
@@ -12362,7 +12362,7 @@
         <v>5</v>
       </c>
       <c r="D7" s="10">
-        <v>-0.124185568588943</v>
+        <v>-0.1109376253507536</v>
       </c>
       <c r="E7" s="10">
         <v>2.965177298596333</v>
@@ -12372,10 +12372,10 @@
         <v>Ya</v>
       </c>
       <c r="G7" s="13">
-        <v>1875628.454717931</v>
+        <v>1854132.454722977</v>
       </c>
       <c r="H7" s="15">
-        <v>0.1568959480812602</v>
+        <v>0.1562738550747418</v>
       </c>
       <c r="I7" s="15">
         <v>0.2900364862563782</v>
@@ -20939,7 +20939,7 @@
         <v>213</v>
       </c>
       <c r="B78" s="10">
-        <v>2410.3148</v>
+        <v>3756.805</v>
       </c>
       <c r="C78" t="s">
         <v>209</v>
@@ -21634,17 +21634,17 @@
         <v>269</v>
       </c>
       <c r="C20" s="10">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>270</v>
       </c>
       <c r="E20" s="8">
-        <v>140.3716049382716</v>
+        <v>140.1565217391304</v>
       </c>
       <c r="F20" s="12">
         <f>C20*E20</f>
-        <v>22740.2</v>
+        <v>22565.199999999997</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>271</v>
@@ -21658,17 +21658,17 @@
         <v>272</v>
       </c>
       <c r="C21" s="10">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>270</v>
       </c>
       <c r="E21" s="8">
-        <v>69.90202702702703</v>
+        <v>69.83766233766234</v>
       </c>
       <c r="F21" s="12">
         <f>C21*E21</f>
-        <v>10345.5</v>
+        <v>10755.0</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>271</v>
@@ -21682,17 +21682,17 @@
         <v>273</v>
       </c>
       <c r="C22" s="10">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>270</v>
       </c>
       <c r="E22" s="8">
-        <v>70.40753424657535</v>
+        <v>70.19140625000001</v>
       </c>
       <c r="F22" s="12">
         <f>C22*E22</f>
-        <v>5139.750000000001</v>
+        <v>4492.250000000001</v>
       </c>
       <c r="G22" s="6" t="s">
         <v>271</v>
@@ -21706,17 +21706,17 @@
         <v>274</v>
       </c>
       <c r="C23" s="10">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>270</v>
       </c>
       <c r="E23" s="8">
-        <v>45.12228260869565</v>
+        <v>44.74431818181818</v>
       </c>
       <c r="F23" s="12">
         <f>C23*E23</f>
-        <v>4151.25</v>
+        <v>3937.5</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>271</v>
@@ -21730,17 +21730,17 @@
         <v>275</v>
       </c>
       <c r="C24" s="10">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>270</v>
       </c>
       <c r="E24" s="8">
-        <v>112.8502024291498</v>
+        <v>110.28125</v>
       </c>
       <c r="F24" s="12">
         <f>C24*E24</f>
-        <v>27874.0</v>
+        <v>28232.0</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>271</v>
@@ -21861,11 +21861,11 @@
       </c>
       <c r="E29" s="12">
         <f>SUM(F4:F28)</f>
-        <v>3650314.861385149</v>
+        <v>3650046.111385149</v>
       </c>
       <c r="F29" s="12">
         <f>C29*E29</f>
-        <v>365031.48613851494</v>
+        <v>365004.61113851494</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>287</v>
@@ -21886,7 +21886,7 @@
       </c>
       <c r="F32" s="3">
         <f>SUM(F4:F29)</f>
-        <v>4015346.3475236637</v>
+        <v>4015050.7225236637</v>
       </c>
     </row>
     <row r="33" spans="2:6">
@@ -21895,7 +21895,7 @@
       </c>
       <c r="F33" s="3">
         <f>FCI26*(1+a_infl)^(a_year0-2026)</f>
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
     </row>
     <row r="34" spans="2:6">
@@ -21904,7 +21904,7 @@
       </c>
       <c r="F34" s="3">
         <f>SUM(F4:F25)*(1+a_cont)*(1+a_infl)^(a_year0-2026)</f>
-        <v>3808025.55811145</v>
+        <v>3807724.02061145</v>
       </c>
     </row>
     <row r="35" spans="2:6">
@@ -21913,7 +21913,7 @@
       </c>
       <c r="F35" s="3">
         <f>FCI26/t_P_gross</f>
-        <v>3564.1810183390016</v>
+        <v>3563.918609838625</v>
       </c>
     </row>
     <row r="36" spans="2:6">
@@ -21922,7 +21922,7 @@
       </c>
       <c r="F36" s="3">
         <f>a_debt_frac*FCI*a_r_debt*0.5</f>
-        <v>98295.67858737928</v>
+        <v>98288.44168737928</v>
       </c>
     </row>
     <row r="37" spans="2:6">
@@ -21931,7 +21931,7 @@
       </c>
       <c r="F37" s="3">
         <f>a_debt_frac*FCI+IDC</f>
-        <v>2555687.6432718616</v>
+        <v>2555499.4838718614</v>
       </c>
     </row>
     <row r="38" spans="2:6">
@@ -21940,7 +21940,7 @@
       </c>
       <c r="F38" s="3">
         <f>DEBT*a_r_debt/(1-(1+a_r_debt)^-(a_tenor-1))</f>
-        <v>409113.7346694201</v>
+        <v>409083.6141673901</v>
       </c>
     </row>
     <row r="40" spans="2:6">
@@ -22048,7 +22048,7 @@
       </c>
       <c r="B8" s="12">
         <f>a_c_ins*FCI26</f>
-        <v>20076.73173761832</v>
+        <v>20075.25361261832</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>303</v>
@@ -22078,7 +22078,7 @@
       </c>
       <c r="B10" s="12">
         <f>a_lease*t_plot_m2</f>
-        <v>4820.6296</v>
+        <v>7513.61</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>303</v>
@@ -22093,7 +22093,7 @@
       </c>
       <c r="B12" s="3">
         <f>B4+B6+B8+B9+B10</f>
-        <v>177481.59079771547</v>
+        <v>180173.09307271548</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -23411,83 +23411,83 @@
       </c>
       <c r="D18" s="13">
         <f>IF(D4=0,0,-(OPEX_F+OPEX_V*D7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(D5-2026))</f>
-        <v>-283730.9874073871</v>
+        <v>-286531.2263742971</v>
       </c>
       <c r="E18" s="13">
         <f>IF(E4=0,0,-(OPEX_F+OPEX_V*E7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(E5-2026))</f>
-        <v>-332717.3456476518</v>
+        <v>-335573.58939390007</v>
       </c>
       <c r="F18" s="13">
         <f>IF(F4=0,0,-(OPEX_F+OPEX_V*F7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(F5-2026))</f>
-        <v>-339371.6925606048</v>
+        <v>-342285.061181778</v>
       </c>
       <c r="G18" s="13">
         <f>IF(G4=0,0,-(OPEX_F+OPEX_V*G7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(G5-2026))</f>
-        <v>-346159.1264118169</v>
+        <v>-349130.76240541355</v>
       </c>
       <c r="H18" s="13">
         <f>IF(H4=0,0,-(OPEX_F+OPEX_V*H7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(H5-2026))</f>
-        <v>-353082.3089400533</v>
+        <v>-356113.37765352183</v>
       </c>
       <c r="I18" s="13">
         <f>IF(I4=0,0,-(OPEX_F+OPEX_V*I7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(I5-2026))</f>
-        <v>-360143.9551188543</v>
+        <v>-363235.6452065923</v>
       </c>
       <c r="J18" s="13">
         <f>IF(J4=0,0,-(OPEX_F+OPEX_V*J7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(J5-2026))</f>
-        <v>-367346.8342212314</v>
+        <v>-370500.35811072413</v>
       </c>
       <c r="K18" s="13">
         <f>IF(K4=0,0,-(OPEX_F+OPEX_V*K7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(K5-2026))</f>
-        <v>-374693.77090565604</v>
+        <v>-377910.3652729386</v>
       </c>
       <c r="L18" s="13">
         <f>IF(L4=0,0,-(OPEX_F+OPEX_V*L7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(L5-2026))</f>
-        <v>-382187.6463237692</v>
+        <v>-385468.5725783974</v>
       </c>
       <c r="M18" s="13">
         <f>IF(M4=0,0,-(OPEX_F+OPEX_V*M7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(M5-2026))</f>
-        <v>-389831.39925024455</v>
+        <v>-393177.9440299654</v>
       </c>
       <c r="N18" s="13">
         <f>IF(N4=0,0,-(OPEX_F+OPEX_V*N7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(N5-2026))</f>
-        <v>-397628.02723524946</v>
+        <v>-401041.50291056465</v>
       </c>
       <c r="O18" s="13">
         <f>IF(O4=0,0,-(OPEX_F+OPEX_V*O7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(O5-2026))</f>
-        <v>-405580.5877799545</v>
+        <v>-409062.332968776</v>
       </c>
       <c r="P18" s="13">
         <f>IF(P4=0,0,-(OPEX_F+OPEX_V*P7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(P5-2026))</f>
-        <v>-413692.1995355535</v>
+        <v>-417243.5796281515</v>
       </c>
       <c r="Q18" s="13">
         <f>IF(Q4=0,0,-(OPEX_F+OPEX_V*Q7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(Q5-2026))</f>
-        <v>-421966.04352626466</v>
+        <v>-425588.45122071455</v>
       </c>
       <c r="R18" s="13">
         <f>IF(R4=0,0,-(OPEX_F+OPEX_V*R7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(R5-2026))</f>
-        <v>-430405.3643967899</v>
+        <v>-434100.22024512885</v>
       </c>
       <c r="S18" s="13">
         <f>IF(S4=0,0,-(OPEX_F+OPEX_V*S7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(S5-2026))</f>
-        <v>-439013.4716847258</v>
+        <v>-442782.2246500315</v>
       </c>
       <c r="T18" s="13">
         <f>IF(T4=0,0,-(OPEX_F+OPEX_V*T7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(T5-2026))</f>
-        <v>-447793.7411184203</v>
+        <v>-451637.8691430321</v>
       </c>
       <c r="U18" s="13">
         <f>IF(U4=0,0,-(OPEX_F+OPEX_V*U7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(U5-2026))</f>
-        <v>-456749.6159407887</v>
+        <v>-460670.6265258927</v>
       </c>
       <c r="V18" s="13">
         <f>IF(V4=0,0,-(OPEX_F+OPEX_V*V7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(V5-2026))</f>
-        <v>-465884.6082596045</v>
+        <v>-469884.0390564106</v>
       </c>
       <c r="W18" s="13">
         <f>IF(W4=0,0,-(OPEX_F+OPEX_V*W7/(t_E_year*a_util/t_up*a_avail))*(1+a_infl)^(W5-2026))</f>
-        <v>-475202.30042479653</v>
+        <v>-479281.7198375388</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -23589,83 +23589,83 @@
       </c>
       <c r="D20" s="14">
         <f>D17+D18+D19</f>
-        <v>388977.70661546063</v>
+        <v>386177.46764855064</v>
       </c>
       <c r="E20" s="14">
         <f>E17+E18+E19</f>
-        <v>683382.9522637548</v>
+        <v>680526.7085175066</v>
       </c>
       <c r="F20" s="14">
         <f>F17+F18+F19</f>
-        <v>721426.3945163141</v>
+        <v>718513.0258951411</v>
       </c>
       <c r="G20" s="14">
         <f>G17+G18+G19</f>
-        <v>726916.988655982</v>
+        <v>723945.3526623853</v>
       </c>
       <c r="H20" s="14">
         <f>H17+H18+H19</f>
-        <v>732517.3946784432</v>
+        <v>729486.3259649747</v>
       </c>
       <c r="I20" s="14">
         <f>I17+I18+I19</f>
-        <v>738229.8088213538</v>
+        <v>735138.1187336158</v>
       </c>
       <c r="J20" s="14">
         <f>J17+J18+J19</f>
-        <v>744056.4712471225</v>
+        <v>740902.9473576298</v>
       </c>
       <c r="K20" s="14">
         <f>K17+K18+K19</f>
-        <v>749999.6669214066</v>
+        <v>746783.072554124</v>
       </c>
       <c r="L20" s="14">
         <f>L17+L18+L19</f>
-        <v>756061.7265091764</v>
+        <v>752780.8002545482</v>
       </c>
       <c r="M20" s="14">
         <f>M17+M18+M19</f>
-        <v>762245.0272887016</v>
+        <v>758898.4825089808</v>
       </c>
       <c r="N20" s="14">
         <f>N17+N18+N19</f>
-        <v>614963.1254934758</v>
+        <v>611549.6498181606</v>
       </c>
       <c r="O20" s="14">
         <f>O17+O18+O19</f>
-        <v>528051.1551182314</v>
+        <v>524569.40992941</v>
       </c>
       <c r="P20" s="14">
         <f>P17+P18+P19</f>
-        <v>534923.3889631787</v>
+        <v>531372.0088705808</v>
       </c>
       <c r="Q20" s="14">
         <f>Q17+Q18+Q19</f>
-        <v>541933.0674850249</v>
+        <v>538310.659790575</v>
       </c>
       <c r="R20" s="14">
         <f>R17+R18+R19</f>
-        <v>549082.9395773081</v>
+        <v>545388.0837289692</v>
       </c>
       <c r="S20" s="14">
         <f>S17+S18+S19</f>
-        <v>556375.8091114368</v>
+        <v>552607.0561461311</v>
       </c>
       <c r="T20" s="14">
         <f>T17+T18+T19</f>
-        <v>563814.5360362481</v>
+        <v>559970.4080116363</v>
       </c>
       <c r="U20" s="14">
         <f>U17+U18+U19</f>
-        <v>571402.0374995556</v>
+        <v>567481.0269144517</v>
       </c>
       <c r="V20" s="14">
         <f>V17+V18+V19</f>
-        <v>579141.2889921295</v>
+        <v>575141.8581953235</v>
       </c>
       <c r="W20" s="14">
         <f>W17+W18+W19</f>
-        <v>587035.3255145547</v>
+        <v>582955.9061018125</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -23674,7 +23674,7 @@
       </c>
       <c r="C21" s="13">
         <f>IF(C4=0,-FCI,0)</f>
-        <v>-4095653.274474137</v>
+        <v>-4095351.736974137</v>
       </c>
       <c r="D21" s="13">
         <f>IF(D4=0,-FCI,0)</f>
@@ -23852,7 +23852,7 @@
       </c>
       <c r="C23" s="13">
         <f>IF(C4=0,-a_vat*FCI,IF(C4=2,a_vat*FCI,0))</f>
-        <v>-450521.86019215506</v>
+        <v>-450488.69106715504</v>
       </c>
       <c r="D23" s="13">
         <f>IF(D4=0,-a_vat*FCI,IF(D4=2,a_vat*FCI,0))</f>
@@ -23860,7 +23860,7 @@
       </c>
       <c r="E23" s="13">
         <f>IF(E4=0,-a_vat*FCI,IF(E4=2,a_vat*FCI,0))</f>
-        <v>450521.86019215506</v>
+        <v>450488.69106715504</v>
       </c>
       <c r="F23" s="13">
         <f>IF(F4=0,-a_vat*FCI,IF(F4=2,a_vat*FCI,0))</f>
@@ -23945,79 +23945,79 @@
       </c>
       <c r="D24" s="13">
         <f>D17*a_rec_days/365+(D18+D19)*a_pay_days/365</f>
-        <v>91280.97539492944</v>
+        <v>91050.81876751219</v>
       </c>
       <c r="E24" s="13">
         <f>E17*a_rec_days/365+(E18+E19)*a_pay_days/365</f>
-        <v>140730.22571302697</v>
+        <v>140495.46595306136</v>
       </c>
       <c r="F24" s="13">
         <f>F17*a_rec_days/365+(F18+F19)*a_pay_days/365</f>
-        <v>147551.8082887589</v>
+        <v>147312.353333594</v>
       </c>
       <c r="G24" s="13">
         <f>G17*a_rec_days/365+(G18+G19)*a_pay_days/365</f>
-        <v>149033.5950708642</v>
+        <v>148789.35101659596</v>
       </c>
       <c r="H24" s="13">
         <f>H17*a_rec_days/365+(H18+H19)*a_pay_days/365</f>
-        <v>150545.0175886116</v>
+        <v>150295.88865325804</v>
       </c>
       <c r="I24" s="13">
         <f>I17*a_rec_days/365+(I18+I19)*a_pay_days/365</f>
-        <v>152086.66855671396</v>
+        <v>151832.5570426533</v>
       </c>
       <c r="J24" s="13">
         <f>J17*a_rec_days/365+(J18+J19)*a_pay_days/365</f>
-        <v>153659.1525441784</v>
+        <v>153399.95879983652</v>
       </c>
       <c r="K24" s="13">
         <f>K17*a_rec_days/365+(K18+K19)*a_pay_days/365</f>
-        <v>155263.0862113921</v>
+        <v>154998.7085921634</v>
       </c>
       <c r="L24" s="13">
         <f>L17*a_rec_days/365+(L18+L19)*a_pay_days/365</f>
-        <v>156899.09855195007</v>
+        <v>156629.4333803368</v>
       </c>
       <c r="M24" s="13">
         <f>M17*a_rec_days/365+(M18+M19)*a_pay_days/365</f>
-        <v>158567.83113931917</v>
+        <v>158292.77266427362</v>
       </c>
       <c r="N24" s="13">
         <f>N17*a_rec_days/365+(N18+N19)*a_pay_days/365</f>
-        <v>135022.45313070834</v>
+        <v>134741.8934861619</v>
       </c>
       <c r="O24" s="13">
         <f>O17*a_rec_days/365+(O18+O19)*a_pay_days/365</f>
-        <v>120138.320384911</v>
+        <v>119852.14954747361</v>
       </c>
       <c r="P24" s="13">
         <f>P17*a_rec_days/365+(P18+P19)*a_pay_days/365</f>
-        <v>121934.71047632146</v>
+        <v>121642.81622213533</v>
       </c>
       <c r="Q24" s="13">
         <f>Q17*a_rec_days/365+(Q18+Q19)*a_pay_days/365</f>
-        <v>123767.0283695601</v>
+        <v>123469.29623029025</v>
       </c>
       <c r="R24" s="13">
         <f>R17*a_rec_days/365+(R18+R19)*a_pay_days/365</f>
-        <v>125635.99262066353</v>
+        <v>125332.30583860827</v>
       </c>
       <c r="S24" s="13">
         <f>S17*a_rec_days/365+(S18+S19)*a_pay_days/365</f>
-        <v>127542.336156789</v>
+        <v>127232.57563909263</v>
       </c>
       <c r="T24" s="13">
         <f>T17*a_rec_days/365+(T18+T19)*a_pay_days/365</f>
-        <v>129486.80656363696</v>
+        <v>129170.85083558668</v>
       </c>
       <c r="U24" s="13">
         <f>U17*a_rec_days/365+(U18+U19)*a_pay_days/365</f>
-        <v>131470.1663786219</v>
+        <v>131147.89153601063</v>
       </c>
       <c r="V24" s="13">
         <f>V17*a_rec_days/365+(V18+V19)*a_pay_days/365</f>
-        <v>133493.1933899066</v>
+        <v>133164.47305044308</v>
       </c>
       <c r="W24" s="13">
         <v>0</v>
@@ -24033,83 +24033,83 @@
       </c>
       <c r="D25" s="13">
         <f>-(D24-C24)</f>
-        <v>-91280.97539492944</v>
+        <v>-91050.81876751219</v>
       </c>
       <c r="E25" s="13">
         <f>-(E24-D24)</f>
-        <v>-49449.25031809753</v>
+        <v>-49444.64718554917</v>
       </c>
       <c r="F25" s="13">
         <f>-(F24-E24)</f>
-        <v>-6821.58257573194</v>
+        <v>-6816.887380532629</v>
       </c>
       <c r="G25" s="13">
         <f>-(G24-F24)</f>
-        <v>-1481.7867821052787</v>
+        <v>-1476.9976830019732</v>
       </c>
       <c r="H25" s="13">
         <f>-(H24-G24)</f>
-        <v>-1511.4225177474145</v>
+        <v>-1506.5376366620767</v>
       </c>
       <c r="I25" s="13">
         <f>-(I24-H24)</f>
-        <v>-1541.65096810236</v>
+        <v>-1536.6683893952577</v>
       </c>
       <c r="J25" s="13">
         <f>-(J24-I24)</f>
-        <v>-1572.483987464424</v>
+        <v>-1567.4017571832228</v>
       </c>
       <c r="K25" s="13">
         <f>-(K24-J24)</f>
-        <v>-1603.9336672137142</v>
+        <v>-1598.749792326882</v>
       </c>
       <c r="L25" s="13">
         <f>-(L24-K24)</f>
-        <v>-1636.0123405579652</v>
+        <v>-1630.7247881733929</v>
       </c>
       <c r="M25" s="13">
         <f>-(M24-L24)</f>
-        <v>-1668.7325873691007</v>
+        <v>-1663.3392839368316</v>
       </c>
       <c r="N25" s="13">
         <f>-(N24-M24)</f>
-        <v>23545.37800861083</v>
+        <v>23550.879178111732</v>
       </c>
       <c r="O25" s="13">
         <f>-(O24-N24)</f>
-        <v>14884.132745797338</v>
+        <v>14889.743938688276</v>
       </c>
       <c r="P25" s="13">
         <f>-(P24-O24)</f>
-        <v>-1796.3900914104597</v>
+        <v>-1790.666674661712</v>
       </c>
       <c r="Q25" s="13">
         <f>-(Q24-P24)</f>
-        <v>-1832.3178932386363</v>
+        <v>-1826.4800081549183</v>
       </c>
       <c r="R25" s="13">
         <f>-(R24-Q24)</f>
-        <v>-1868.9642511034326</v>
+        <v>-1863.0096083180251</v>
       </c>
       <c r="S25" s="13">
         <f>-(S24-R24)</f>
-        <v>-1906.343536125467</v>
+        <v>-1900.269800484355</v>
       </c>
       <c r="T25" s="13">
         <f>-(T24-S24)</f>
-        <v>-1944.4704068479623</v>
+        <v>-1938.2751964940544</v>
       </c>
       <c r="U25" s="13">
         <f>-(U24-T24)</f>
-        <v>-1983.3598149849568</v>
+        <v>-1977.0407004239532</v>
       </c>
       <c r="V25" s="13">
         <f>-(V24-U24)</f>
-        <v>-2023.027011284692</v>
+        <v>-2016.5815144324442</v>
       </c>
       <c r="W25" s="13">
         <f>-(W24-V24)</f>
-        <v>133493.1933899066</v>
+        <v>133164.47305044308</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -24121,35 +24121,35 @@
       </c>
       <c r="D26" s="13">
         <f>IF(D4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:D22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="E26" s="13">
         <f>IF(E4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:E22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="F26" s="13">
         <f>IF(F4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:F22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="G26" s="13">
         <f>IF(G4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:G22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="H26" s="13">
         <f>IF(H4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:H22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="I26" s="13">
         <f>IF(I4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:I22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="J26" s="13">
         <f>IF(J4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:J22)/8</f>
-        <v>524243.61913268955</v>
+        <v>524205.02233268955</v>
       </c>
       <c r="K26" s="13">
         <f>IF(K4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(D22:K22)/8</f>
-        <v>551133.2019266916</v>
+        <v>551094.6051266915</v>
       </c>
       <c r="L26" s="13">
         <f>IF(L4&lt;=a_dep_life,(FCI+IDC)/a_dep_life,0)-SUM(E22:L22)/8</f>
@@ -24210,27 +24210,27 @@
       </c>
       <c r="D27" s="13">
         <f>IF(AND(D4&gt;=1,D4&lt;=6),a_allow*TANG/6,0)</f>
-        <v>190401.27790557253</v>
+        <v>190386.2010305725</v>
       </c>
       <c r="E27" s="13">
         <f>IF(AND(E4&gt;=1,E4&lt;=6),a_allow*TANG/6,0)</f>
-        <v>190401.27790557253</v>
+        <v>190386.2010305725</v>
       </c>
       <c r="F27" s="13">
         <f>IF(AND(F4&gt;=1,F4&lt;=6),a_allow*TANG/6,0)</f>
-        <v>190401.27790557253</v>
+        <v>190386.2010305725</v>
       </c>
       <c r="G27" s="13">
         <f>IF(AND(G4&gt;=1,G4&lt;=6),a_allow*TANG/6,0)</f>
-        <v>190401.27790557253</v>
+        <v>190386.2010305725</v>
       </c>
       <c r="H27" s="13">
         <f>IF(AND(H4&gt;=1,H4&lt;=6),a_allow*TANG/6,0)</f>
-        <v>190401.27790557253</v>
+        <v>190386.2010305725</v>
       </c>
       <c r="I27" s="13">
         <f>IF(AND(I4&gt;=1,I4&lt;=6),a_allow*TANG/6,0)</f>
-        <v>190401.27790557253</v>
+        <v>190386.2010305725</v>
       </c>
       <c r="J27" s="13">
         <f>IF(AND(J4&gt;=1,J4&lt;=6),a_allow*TANG/6,0)</f>
@@ -24299,83 +24299,83 @@
       </c>
       <c r="D28" s="13">
         <f>D20-D26-D27</f>
-        <v>-325667.1904228014</v>
+        <v>-328413.7557147114</v>
       </c>
       <c r="E28" s="13">
         <f>E20-E26-E27</f>
-        <v>-31261.944774507283</v>
+        <v>-34064.514845755446</v>
       </c>
       <c r="F28" s="13">
         <f>F20-F26-F27</f>
-        <v>6781.4974780520715</v>
+        <v>3921.802531879017</v>
       </c>
       <c r="G28" s="13">
         <f>G20-G26-G27</f>
-        <v>12272.091617719881</v>
+        <v>9354.129299123277</v>
       </c>
       <c r="H28" s="13">
         <f>H20-H26-H27</f>
-        <v>17872.49764018113</v>
+        <v>14895.102601712657</v>
       </c>
       <c r="I28" s="13">
         <f>I20-I26-I27</f>
-        <v>23584.911783091753</v>
+        <v>20546.8953703538</v>
       </c>
       <c r="J28" s="13">
         <f>J20-J26-J27</f>
-        <v>219812.85211443296</v>
+        <v>216697.92502494022</v>
       </c>
       <c r="K28" s="13">
         <f>K20-K26-K27</f>
-        <v>198866.46499471506</v>
+        <v>195688.46742743254</v>
       </c>
       <c r="L28" s="13">
         <f>L20-L26-L27</f>
-        <v>729172.1437151744</v>
+        <v>725891.2174605462</v>
       </c>
       <c r="M28" s="13">
         <f>M20-M26-M27</f>
-        <v>735355.4444946996</v>
+        <v>732008.8997149788</v>
       </c>
       <c r="N28" s="13">
         <f>N20-N26-N27</f>
-        <v>588073.5426994738</v>
+        <v>584660.0670241585</v>
       </c>
       <c r="O28" s="13">
         <f>O20-O26-O27</f>
-        <v>489034.01016372506</v>
+        <v>485552.2649749036</v>
       </c>
       <c r="P28" s="13">
         <f>P20-P26-P27</f>
-        <v>495906.24400867237</v>
+        <v>492354.86391607445</v>
       </c>
       <c r="Q28" s="13">
         <f>Q20-Q26-Q27</f>
-        <v>502915.92253051855</v>
+        <v>499293.5148360687</v>
       </c>
       <c r="R28" s="13">
         <f>R20-R26-R27</f>
-        <v>510065.79462280177</v>
+        <v>506370.93877446285</v>
       </c>
       <c r="S28" s="13">
         <f>S20-S26-S27</f>
-        <v>512742.81501910294</v>
+        <v>508974.06205379724</v>
       </c>
       <c r="T28" s="13">
         <f>T20-T26-T27</f>
-        <v>520181.5419439142</v>
+        <v>516337.41391930246</v>
       </c>
       <c r="U28" s="13">
         <f>U20-U26-U27</f>
-        <v>527769.0434072217</v>
+        <v>523848.03282211785</v>
       </c>
       <c r="V28" s="13">
         <f>V20-V26-V27</f>
-        <v>535508.2948997956</v>
+        <v>531508.8641029896</v>
       </c>
       <c r="W28" s="13">
         <f>W20-W26-W27</f>
-        <v>555529.8935827252</v>
+        <v>551450.474169983</v>
       </c>
     </row>
     <row r="29" spans="1:23">
@@ -24505,55 +24505,55 @@
       </c>
       <c r="K30" s="13">
         <f>-a_tax*MAX(0,K28-J29)</f>
-        <v>-26897.45969479449</v>
+        <v>-21697.731372894457</v>
       </c>
       <c r="L30" s="13">
         <f>-a_tax*MAX(0,L28-K29)</f>
-        <v>-160417.87161733836</v>
+        <v>-159696.06784132015</v>
       </c>
       <c r="M30" s="13">
         <f>-a_tax*MAX(0,M28-L29)</f>
-        <v>-161778.1977888339</v>
+        <v>-161041.95793729532</v>
       </c>
       <c r="N30" s="13">
         <f>-a_tax*MAX(0,N28-M29)</f>
-        <v>-129376.17939388423</v>
+        <v>-128625.21474531488</v>
       </c>
       <c r="O30" s="13">
         <f>-a_tax*MAX(0,O28-N29)</f>
-        <v>-107587.48223601951</v>
+        <v>-106821.49829447879</v>
       </c>
       <c r="P30" s="13">
         <f>-a_tax*MAX(0,P28-O29)</f>
-        <v>-109099.37368190792</v>
+        <v>-108318.07006153637</v>
       </c>
       <c r="Q30" s="13">
         <f>-a_tax*MAX(0,Q28-P29)</f>
-        <v>-110641.50295671409</v>
+        <v>-109844.5732639351</v>
       </c>
       <c r="R30" s="13">
         <f>-a_tax*MAX(0,R28-Q29)</f>
-        <v>-112214.4748170164</v>
+        <v>-111401.60653038183</v>
       </c>
       <c r="S30" s="13">
         <f>-a_tax*MAX(0,S28-R29)</f>
-        <v>-112803.41930420265</v>
+        <v>-111974.2936518354</v>
       </c>
       <c r="T30" s="13">
         <f>-a_tax*MAX(0,T28-S29)</f>
-        <v>-114439.93922766112</v>
+        <v>-113594.23106224654</v>
       </c>
       <c r="U30" s="13">
         <f>-a_tax*MAX(0,U28-T29)</f>
-        <v>-116109.18954958877</v>
+        <v>-115246.56722086592</v>
       </c>
       <c r="V30" s="13">
         <f>-a_tax*MAX(0,V28-U29)</f>
-        <v>-117811.82487795502</v>
+        <v>-116931.9501026577</v>
       </c>
       <c r="W30" s="13">
         <f>-a_tax*MAX(0,W28-V29)</f>
-        <v>-122216.57658819955</v>
+        <v>-121319.10431739625</v>
       </c>
     </row>
     <row r="31" spans="1:23">
@@ -24562,87 +24562,87 @@
       </c>
       <c r="C31" s="14">
         <f>C20+C30+C21+C22+C23+C25</f>
-        <v>-4546175.134666292</v>
+        <v>-4545840.428041292</v>
       </c>
       <c r="D31" s="14">
         <f>D20+D30+D21+D22+D23+D25</f>
-        <v>297696.73122053116</v>
+        <v>295126.6488810384</v>
       </c>
       <c r="E31" s="14">
         <f>E20+E30+E21+E22+E23+E25</f>
-        <v>1084455.5621378124</v>
+        <v>1081570.7523991126</v>
       </c>
       <c r="F31" s="14">
         <f>F20+F30+F21+F22+F23+F25</f>
-        <v>714604.8119405822</v>
+        <v>711696.1385146084</v>
       </c>
       <c r="G31" s="14">
         <f>G20+G30+G21+G22+G23+G25</f>
-        <v>725435.2018738766</v>
+        <v>722468.3549793833</v>
       </c>
       <c r="H31" s="14">
         <f>H20+H30+H21+H22+H23+H25</f>
-        <v>731005.9721606958</v>
+        <v>727979.7883283126</v>
       </c>
       <c r="I31" s="14">
         <f>I20+I30+I21+I22+I23+I25</f>
-        <v>736688.1578532514</v>
+        <v>733601.4503442206</v>
       </c>
       <c r="J31" s="14">
         <f>J20+J30+J21+J22+J23+J25</f>
-        <v>742483.987259658</v>
+        <v>739335.5456004465</v>
       </c>
       <c r="K31" s="14">
         <f>K20+K30+K21+K22+K23+K25</f>
-        <v>506381.61120738246</v>
+        <v>508369.9290368867</v>
       </c>
       <c r="L31" s="14">
         <f>L20+L30+L21+L22+L23+L25</f>
-        <v>594007.84255128</v>
+        <v>591454.0076250546</v>
       </c>
       <c r="M31" s="14">
         <f>M20+M30+M21+M22+M23+M25</f>
-        <v>598798.0969124986</v>
+        <v>596193.1852877487</v>
       </c>
       <c r="N31" s="14">
         <f>N20+N30+N21+N22+N23+N25</f>
-        <v>509132.32410820236</v>
+        <v>506475.3142509574</v>
       </c>
       <c r="O31" s="14">
         <f>O20+O30+O21+O22+O23+O25</f>
-        <v>338327.3083439745</v>
+        <v>335617.1582895847</v>
       </c>
       <c r="P31" s="14">
         <f>P20+P30+P21+P22+P23+P25</f>
-        <v>424027.62518986035</v>
+        <v>421263.27213438274</v>
       </c>
       <c r="Q31" s="14">
         <f>Q20+Q30+Q21+Q22+Q23+Q25</f>
-        <v>429459.2466350722</v>
+        <v>426639.606518485</v>
       </c>
       <c r="R31" s="14">
         <f>R20+R30+R21+R22+R23+R25</f>
-        <v>434999.5005091883</v>
+        <v>432123.46759026934</v>
       </c>
       <c r="S31" s="14">
         <f>S20+S30+S21+S22+S23+S25</f>
-        <v>189622.59081647222</v>
+        <v>186689.03723917488</v>
       </c>
       <c r="T31" s="14">
         <f>T20+T30+T21+T22+T23+T25</f>
-        <v>447430.126401739</v>
+        <v>444437.90175289573</v>
       </c>
       <c r="U31" s="14">
         <f>U20+U30+U21+U22+U23+U25</f>
-        <v>453309.4881349819</v>
+        <v>450257.4189931619</v>
       </c>
       <c r="V31" s="14">
         <f>V20+V30+V21+V22+V23+V25</f>
-        <v>459306.43710288976</v>
+        <v>456193.32657823333</v>
       </c>
       <c r="W31" s="14">
         <f>W20+W30+W21+W22+W23+W25</f>
-        <v>598311.9423162618</v>
+        <v>594801.2748348593</v>
       </c>
     </row>
     <row r="32" spans="1:23">
@@ -24651,87 +24651,87 @@
       </c>
       <c r="C32" s="13">
         <f>C31</f>
-        <v>-4546175.134666292</v>
+        <v>-4545840.428041292</v>
       </c>
       <c r="D32" s="13">
         <f>C32+D31</f>
-        <v>-4248478.403445761</v>
+        <v>-4250713.779160254</v>
       </c>
       <c r="E32" s="13">
         <f>D32+E31</f>
-        <v>-3164022.8413079483</v>
+        <v>-3169143.026761141</v>
       </c>
       <c r="F32" s="13">
         <f>E32+F31</f>
-        <v>-2449418.029367366</v>
+        <v>-2457446.8882465325</v>
       </c>
       <c r="G32" s="13">
         <f>F32+G31</f>
-        <v>-1723982.8274934893</v>
+        <v>-1734978.5332671492</v>
       </c>
       <c r="H32" s="13">
         <f>G32+H31</f>
-        <v>-992976.8553327934</v>
+        <v>-1006998.7449388367</v>
       </c>
       <c r="I32" s="13">
         <f>H32+I31</f>
-        <v>-256288.697479542</v>
+        <v>-273397.29459461605</v>
       </c>
       <c r="J32" s="13">
         <f>I32+J31</f>
-        <v>486195.28978011606</v>
+        <v>465938.2510058305</v>
       </c>
       <c r="K32" s="13">
         <f>J32+K31</f>
-        <v>992576.9009874985</v>
+        <v>974308.1800427171</v>
       </c>
       <c r="L32" s="13">
         <f>K32+L31</f>
-        <v>1586584.7435387785</v>
+        <v>1565762.1876677717</v>
       </c>
       <c r="M32" s="13">
         <f>L32+M31</f>
-        <v>2185382.840451277</v>
+        <v>2161955.3729555206</v>
       </c>
       <c r="N32" s="13">
         <f>M32+N31</f>
-        <v>2694515.1645594793</v>
+        <v>2668430.687206478</v>
       </c>
       <c r="O32" s="13">
         <f>N32+O31</f>
-        <v>3032842.4729034537</v>
+        <v>3004047.8454960627</v>
       </c>
       <c r="P32" s="13">
         <f>O32+P31</f>
-        <v>3456870.098093314</v>
+        <v>3425311.1176304454</v>
       </c>
       <c r="Q32" s="13">
         <f>P32+Q31</f>
-        <v>3886329.3447283865</v>
+        <v>3851950.7241489305</v>
       </c>
       <c r="R32" s="13">
         <f>Q32+R31</f>
-        <v>4321328.845237575</v>
+        <v>4284074.1917392</v>
       </c>
       <c r="S32" s="13">
         <f>R32+S31</f>
-        <v>4510951.436054047</v>
+        <v>4470763.228978375</v>
       </c>
       <c r="T32" s="13">
         <f>S32+T31</f>
-        <v>4958381.562455786</v>
+        <v>4915201.130731271</v>
       </c>
       <c r="U32" s="13">
         <f>T32+U31</f>
-        <v>5411691.050590768</v>
+        <v>5365458.549724433</v>
       </c>
       <c r="V32" s="13">
         <f>U32+V31</f>
-        <v>5870997.487693658</v>
+        <v>5821651.876302666</v>
       </c>
       <c r="W32" s="13">
         <f>V32+W31</f>
-        <v>6469309.43000992</v>
+        <v>6416453.151137525</v>
       </c>
     </row>
     <row r="33" spans="1:23">
@@ -24829,87 +24829,87 @@
       </c>
       <c r="C34" s="13">
         <f>C31*C33</f>
-        <v>-4546175.134666292</v>
+        <v>-4545840.428041292</v>
       </c>
       <c r="D34" s="13">
         <f>D31*D33</f>
-        <v>271264.6989544131</v>
+        <v>268922.8102502537</v>
       </c>
       <c r="E34" s="13">
         <f>E31*E33</f>
-        <v>900430.4839356351</v>
+        <v>898035.2077069263</v>
       </c>
       <c r="F34" s="13">
         <f>F31*F33</f>
-        <v>540659.1779481687</v>
+        <v>538458.519686246</v>
       </c>
       <c r="G34" s="13">
         <f>G31*G33</f>
-        <v>500121.4526026833</v>
+        <v>498076.0820793189</v>
       </c>
       <c r="H34" s="13">
         <f>H31*H33</f>
-        <v>459215.985359545</v>
+        <v>457314.94481625175</v>
       </c>
       <c r="I34" s="13">
         <f>I31*I33</f>
-        <v>421695.50875396444</v>
+        <v>419928.61365796</v>
       </c>
       <c r="J34" s="13">
         <f>J31*J33</f>
-        <v>387276.9000104724</v>
+        <v>385634.6844926085</v>
       </c>
       <c r="K34" s="13">
         <f>K31*K33</f>
-        <v>240675.3666864488</v>
+        <v>241620.38347243387</v>
       </c>
       <c r="L34" s="13">
         <f>L31*L33</f>
-        <v>257255.76107271962</v>
+        <v>256149.73401291104</v>
       </c>
       <c r="M34" s="13">
         <f>M31*M33</f>
-        <v>236304.80697927484</v>
+        <v>235276.8258586626</v>
       </c>
       <c r="N34" s="13">
         <f>N31*N33</f>
-        <v>183080.4747819488</v>
+        <v>182125.03234953838</v>
       </c>
       <c r="O34" s="13">
         <f>O31*O33</f>
-        <v>110858.15015899515</v>
+        <v>109970.12777867491</v>
       </c>
       <c r="P34" s="13">
         <f>P31*P33</f>
-        <v>126602.98338361974</v>
+        <v>125777.62361185395</v>
       </c>
       <c r="Q34" s="13">
         <f>Q31*Q33</f>
-        <v>116839.84192017197</v>
+        <v>116072.72301872759</v>
       </c>
       <c r="R34" s="13">
         <f>R31*R33</f>
-        <v>107839.27899885546</v>
+        <v>107126.29124601862</v>
       </c>
       <c r="S34" s="13">
         <f>S31*S33</f>
-        <v>42834.87538807116</v>
+        <v>42172.199061444124</v>
       </c>
       <c r="T34" s="13">
         <f>T31*T33</f>
-        <v>92098.35410226752</v>
+        <v>91482.43901519252</v>
       </c>
       <c r="U34" s="13">
         <f>U31*U33</f>
-        <v>85023.83110502442</v>
+        <v>84451.37758700388</v>
       </c>
       <c r="V34" s="13">
         <f>V31*V33</f>
-        <v>78499.62954883302</v>
+        <v>77967.57076805143</v>
       </c>
       <c r="W34" s="13">
         <f>W31*W33</f>
-        <v>93177.69464775082</v>
+        <v>92630.96328663919</v>
       </c>
     </row>
     <row r="35" spans="1:23">
@@ -24918,87 +24918,87 @@
       </c>
       <c r="C35" s="13">
         <f>C34</f>
-        <v>-4546175.134666292</v>
+        <v>-4545840.428041292</v>
       </c>
       <c r="D35" s="13">
         <f>C35+D34</f>
-        <v>-4274910.435711879</v>
+        <v>-4276917.617791039</v>
       </c>
       <c r="E35" s="13">
         <f>D35+E34</f>
-        <v>-3374479.951776244</v>
+        <v>-3378882.4100841125</v>
       </c>
       <c r="F35" s="13">
         <f>E35+F34</f>
-        <v>-2833820.7738280753</v>
+        <v>-2840423.8903978663</v>
       </c>
       <c r="G35" s="13">
         <f>F35+G34</f>
-        <v>-2333699.321225392</v>
+        <v>-2342347.8083185474</v>
       </c>
       <c r="H35" s="13">
         <f>G35+H34</f>
-        <v>-1874483.3358658473</v>
+        <v>-1885032.8635022957</v>
       </c>
       <c r="I35" s="13">
         <f>H35+I34</f>
-        <v>-1452787.8271118829</v>
+        <v>-1465104.2498443357</v>
       </c>
       <c r="J35" s="13">
         <f>I35+J34</f>
-        <v>-1065510.9271014105</v>
+        <v>-1079469.5653517272</v>
       </c>
       <c r="K35" s="13">
         <f>J35+K34</f>
-        <v>-824835.5604149617</v>
+        <v>-837849.1818792933</v>
       </c>
       <c r="L35" s="13">
         <f>K35+L34</f>
-        <v>-567579.7993422421</v>
+        <v>-581699.4478663823</v>
       </c>
       <c r="M35" s="13">
         <f>L35+M34</f>
-        <v>-331274.9923629672</v>
+        <v>-346422.6220077197</v>
       </c>
       <c r="N35" s="13">
         <f>M35+N34</f>
-        <v>-148194.51758101842</v>
+        <v>-164297.58965818133</v>
       </c>
       <c r="O35" s="13">
         <f>N35+O34</f>
-        <v>-37336.367422023264</v>
+        <v>-54327.461879506416</v>
       </c>
       <c r="P35" s="13">
         <f>O35+P34</f>
-        <v>89266.61596159647</v>
+        <v>71450.16173234754</v>
       </c>
       <c r="Q35" s="13">
         <f>P35+Q34</f>
-        <v>206106.45788176844</v>
+        <v>187522.88475107512</v>
       </c>
       <c r="R35" s="13">
         <f>Q35+R34</f>
-        <v>313945.7368806239</v>
+        <v>294649.1759970937</v>
       </c>
       <c r="S35" s="13">
         <f>R35+S34</f>
-        <v>356780.6122686951</v>
+        <v>336821.3750585379</v>
       </c>
       <c r="T35" s="13">
         <f>S35+T34</f>
-        <v>448878.9663709626</v>
+        <v>428303.8140737304</v>
       </c>
       <c r="U35" s="13">
         <f>T35+U34</f>
-        <v>533902.797475987</v>
+        <v>512755.19166073424</v>
       </c>
       <c r="V35" s="13">
         <f>U35+V34</f>
-        <v>612402.42702482</v>
+        <v>590722.7624287857</v>
       </c>
       <c r="W35" s="13">
         <f>V35+W34</f>
-        <v>705580.1216725708</v>
+        <v>683353.7257154249</v>
       </c>
     </row>
     <row r="36" spans="1:23">
@@ -25188,43 +25188,43 @@
       </c>
       <c r="D38" s="13">
         <f>IF(D4&lt;=a_tenor,C40*a_r_debt,0)</f>
-        <v>204455.01146174895</v>
+        <v>204439.95870974893</v>
       </c>
       <c r="E38" s="13">
         <f>IF(E4&lt;=a_tenor,D40*a_r_debt,0)</f>
-        <v>204455.01146174895</v>
+        <v>204439.95870974893</v>
       </c>
       <c r="F38" s="13">
         <f>IF(F4&lt;=a_tenor,E40*a_r_debt,0)</f>
-        <v>188082.31360513525</v>
+        <v>188068.46627313763</v>
       </c>
       <c r="G38" s="13">
         <f>IF(G4&lt;=a_tenor,F40*a_r_debt,0)</f>
-        <v>170399.79991999245</v>
+        <v>170387.25444159744</v>
       </c>
       <c r="H38" s="13">
         <f>IF(H4&lt;=a_tenor,G40*a_r_debt,0)</f>
-        <v>151302.68514003826</v>
+        <v>151291.54566353402</v>
       </c>
       <c r="I38" s="13">
         <f>IF(I4&lt;=a_tenor,H40*a_r_debt,0)</f>
-        <v>130677.80117768771</v>
+        <v>130668.18018322554</v>
       </c>
       <c r="J38" s="13">
         <f>IF(J4&lt;=a_tenor,I40*a_r_debt,0)</f>
-        <v>108402.9264983491</v>
+        <v>108394.94546449237</v>
       </c>
       <c r="K38" s="13">
         <f>IF(K4&lt;=a_tenor,J40*a_r_debt,0)</f>
-        <v>84346.06184466343</v>
+        <v>84339.85196826055</v>
       </c>
       <c r="L38" s="13">
         <f>IF(L4&lt;=a_tenor,K40*a_r_debt,0)</f>
-        <v>58364.6480186829</v>
+        <v>58360.35099233019</v>
       </c>
       <c r="M38" s="13">
         <f>IF(M4&lt;=a_tenor,L40*a_r_debt,0)</f>
-        <v>30304.721086623922</v>
+        <v>30302.489938325398</v>
       </c>
       <c r="N38" s="13">
         <f>IF(N4&lt;=a_tenor,M40*a_r_debt,0)</f>
@@ -25280,39 +25280,39 @@
       </c>
       <c r="E39" s="13">
         <f>IF(AND(E4&gt;=2,E4&lt;=a_tenor),ANN-E38,0)</f>
-        <v>204658.72320767117</v>
+        <v>204643.65545764117</v>
       </c>
       <c r="F39" s="13">
         <f>IF(AND(F4&gt;=2,F4&lt;=a_tenor),ANN-F38,0)</f>
-        <v>221031.42106428486</v>
+        <v>221015.14789425247</v>
       </c>
       <c r="G39" s="13">
         <f>IF(AND(G4&gt;=2,G4&lt;=a_tenor),ANN-G38,0)</f>
-        <v>238713.93474942766</v>
+        <v>238696.35972579266</v>
       </c>
       <c r="H39" s="13">
         <f>IF(AND(H4&gt;=2,H4&lt;=a_tenor),ANN-H38,0)</f>
-        <v>257811.04952938185</v>
+        <v>257792.06850385608</v>
       </c>
       <c r="I39" s="13">
         <f>IF(AND(I4&gt;=2,I4&lt;=a_tenor),ANN-I38,0)</f>
-        <v>278435.9334917324</v>
+        <v>278415.43398416456</v>
       </c>
       <c r="J39" s="13">
         <f>IF(AND(J4&gt;=2,J4&lt;=a_tenor),ANN-J38,0)</f>
-        <v>300710.808171071</v>
+        <v>300688.66870289773</v>
       </c>
       <c r="K39" s="13">
         <f>IF(AND(K4&gt;=2,K4&lt;=a_tenor),ANN-K38,0)</f>
-        <v>324767.6728247567</v>
+        <v>324743.76219912956</v>
       </c>
       <c r="L39" s="13">
         <f>IF(AND(L4&gt;=2,L4&lt;=a_tenor),ANN-L38,0)</f>
-        <v>350749.0866507372</v>
+        <v>350723.2631750599</v>
       </c>
       <c r="M39" s="13">
         <f>IF(AND(M4&gt;=2,M4&lt;=a_tenor),ANN-M38,0)</f>
-        <v>378809.0135827962</v>
+        <v>378781.1242290647</v>
       </c>
       <c r="N39" s="13">
         <f>IF(AND(N4&gt;=2,N4&lt;=a_tenor),ANN-N38,0)</f>
@@ -25361,43 +25361,43 @@
       </c>
       <c r="C40" s="13">
         <f>DEBT</f>
-        <v>2555687.6432718616</v>
+        <v>2555499.4838718614</v>
       </c>
       <c r="D40" s="13">
         <f>C40-D39</f>
-        <v>2555687.6432718616</v>
+        <v>2555499.4838718614</v>
       </c>
       <c r="E40" s="13">
         <f>D40-E39</f>
-        <v>2351028.9200641904</v>
+        <v>2350855.8284142204</v>
       </c>
       <c r="F40" s="13">
         <f>E40-F39</f>
-        <v>2129997.498999906</v>
+        <v>2129840.680519968</v>
       </c>
       <c r="G40" s="13">
         <f>F40-G39</f>
-        <v>1891283.564250478</v>
+        <v>1891144.3207941751</v>
       </c>
       <c r="H40" s="13">
         <f>G40-H39</f>
-        <v>1633472.5147210963</v>
+        <v>1633352.2522903192</v>
       </c>
       <c r="I40" s="13">
         <f>H40-I39</f>
-        <v>1355036.5812293638</v>
+        <v>1354936.8183061546</v>
       </c>
       <c r="J40" s="13">
         <f>I40-J39</f>
-        <v>1054325.773058293</v>
+        <v>1054248.149603257</v>
       </c>
       <c r="K40" s="13">
         <f>J40-K39</f>
-        <v>729558.1002335362</v>
+        <v>729504.3874041274</v>
       </c>
       <c r="L40" s="13">
         <f>K40-L39</f>
-        <v>378809.013582799</v>
+        <v>378781.12422906747</v>
       </c>
       <c r="M40" s="13">
         <f>L40-M39</f>
@@ -25450,7 +25450,7 @@
       </c>
       <c r="C41" s="13">
         <f>-a_fee_debt*DEBT</f>
-        <v>-38335.314649077925</v>
+        <v>-38332.49225807792</v>
       </c>
       <c r="D41" s="13">
         <v>0</v>
@@ -25523,7 +25523,7 @@
       </c>
       <c r="D42" s="13">
         <f>IF(D4=1,-ANN*a_dsra_m/12,IF(D4=a_tenor,ANN*a_dsra_m/12,0))</f>
-        <v>-204556.86733471006</v>
+        <v>-204541.80708369505</v>
       </c>
       <c r="E42" s="13">
         <f>IF(E4=1,-ANN*a_dsra_m/12,IF(E4=a_tenor,ANN*a_dsra_m/12,0))</f>
@@ -25559,7 +25559,7 @@
       </c>
       <c r="M42" s="13">
         <f>IF(M4=1,-ANN*a_dsra_m/12,IF(M4=a_tenor,ANN*a_dsra_m/12,0))</f>
-        <v>204556.86733471006</v>
+        <v>204541.80708369505</v>
       </c>
       <c r="N42" s="13">
         <f>IF(N4=1,-ANN*a_dsra_m/12,IF(N4=a_tenor,ANN*a_dsra_m/12,0))</f>
@@ -25612,83 +25612,83 @@
       </c>
       <c r="D43" s="13">
         <f>D28-D38+IF(D4=1,C41,0)</f>
-        <v>-568457.5165336283</v>
+        <v>-571186.2066825383</v>
       </c>
       <c r="E43" s="13">
         <f>E28-E38+IF(E4=1,C41,0)</f>
-        <v>-235716.95623625623</v>
+        <v>-238504.47355550437</v>
       </c>
       <c r="F43" s="13">
         <f>F28-F38+IF(F4=1,C41,0)</f>
-        <v>-181300.81612708318</v>
+        <v>-184146.6637412586</v>
       </c>
       <c r="G43" s="13">
         <f>G28-G38+IF(G4=1,C41,0)</f>
-        <v>-158127.70830227257</v>
+        <v>-161033.12514247416</v>
       </c>
       <c r="H43" s="13">
         <f>H28-H38+IF(H4=1,C41,0)</f>
-        <v>-133430.18749985713</v>
+        <v>-136396.44306182137</v>
       </c>
       <c r="I43" s="13">
         <f>I28-I38+IF(I4=1,C41,0)</f>
-        <v>-107092.88939459596</v>
+        <v>-110121.28481287175</v>
       </c>
       <c r="J43" s="13">
         <f>J28-J38+IF(J4=1,C41,0)</f>
-        <v>111409.92561608386</v>
+        <v>108302.97956044786</v>
       </c>
       <c r="K43" s="13">
         <f>K28-K38+IF(K4=1,C41,0)</f>
-        <v>114520.40315005163</v>
+        <v>111348.61545917198</v>
       </c>
       <c r="L43" s="13">
         <f>L28-L38+IF(L4=1,C41,0)</f>
-        <v>670807.4956964916</v>
+        <v>667530.866468216</v>
       </c>
       <c r="M43" s="13">
         <f>M28-M38+IF(M4=1,C41,0)</f>
-        <v>705050.7234080756</v>
+        <v>701706.4097766534</v>
       </c>
       <c r="N43" s="13">
         <f>N28-N38+IF(N4=1,C41,0)</f>
-        <v>588073.5426994738</v>
+        <v>584660.0670241585</v>
       </c>
       <c r="O43" s="13">
         <f>O28-O38+IF(O4=1,C41,0)</f>
-        <v>489034.01016372506</v>
+        <v>485552.2649749036</v>
       </c>
       <c r="P43" s="13">
         <f>P28-P38+IF(P4=1,C41,0)</f>
-        <v>495906.24400867237</v>
+        <v>492354.86391607445</v>
       </c>
       <c r="Q43" s="13">
         <f>Q28-Q38+IF(Q4=1,C41,0)</f>
-        <v>502915.92253051855</v>
+        <v>499293.5148360687</v>
       </c>
       <c r="R43" s="13">
         <f>R28-R38+IF(R4=1,C41,0)</f>
-        <v>510065.79462280177</v>
+        <v>506370.93877446285</v>
       </c>
       <c r="S43" s="13">
         <f>S28-S38+IF(S4=1,C41,0)</f>
-        <v>512742.81501910294</v>
+        <v>508974.06205379724</v>
       </c>
       <c r="T43" s="13">
         <f>T28-T38+IF(T4=1,C41,0)</f>
-        <v>520181.5419439142</v>
+        <v>516337.41391930246</v>
       </c>
       <c r="U43" s="13">
         <f>U28-U38+IF(U4=1,C41,0)</f>
-        <v>527769.0434072217</v>
+        <v>523848.03282211785</v>
       </c>
       <c r="V43" s="13">
         <f>V28-V38+IF(V4=1,C41,0)</f>
-        <v>535508.2948997956</v>
+        <v>531508.8641029896</v>
       </c>
       <c r="W43" s="13">
         <f>W28-W38+IF(W4=1,C41,0)</f>
-        <v>555529.8935827252</v>
+        <v>551450.474169983</v>
       </c>
     </row>
     <row r="44" spans="1:23">
@@ -25826,47 +25826,47 @@
       </c>
       <c r="M45" s="13">
         <f>-a_tax*MAX(0,M43-L44)</f>
-        <v>-47885.74423094202</v>
+        <v>-41250.148338964544</v>
       </c>
       <c r="N45" s="13">
         <f>-a_tax*MAX(0,N43-M44)</f>
-        <v>-129376.17939388423</v>
+        <v>-128625.21474531488</v>
       </c>
       <c r="O45" s="13">
         <f>-a_tax*MAX(0,O43-N44)</f>
-        <v>-107587.48223601951</v>
+        <v>-106821.49829447879</v>
       </c>
       <c r="P45" s="13">
         <f>-a_tax*MAX(0,P43-O44)</f>
-        <v>-109099.37368190792</v>
+        <v>-108318.07006153637</v>
       </c>
       <c r="Q45" s="13">
         <f>-a_tax*MAX(0,Q43-P44)</f>
-        <v>-110641.50295671409</v>
+        <v>-109844.5732639351</v>
       </c>
       <c r="R45" s="13">
         <f>-a_tax*MAX(0,R43-Q44)</f>
-        <v>-112214.4748170164</v>
+        <v>-111401.60653038183</v>
       </c>
       <c r="S45" s="13">
         <f>-a_tax*MAX(0,S43-R44)</f>
-        <v>-112803.41930420265</v>
+        <v>-111974.2936518354</v>
       </c>
       <c r="T45" s="13">
         <f>-a_tax*MAX(0,T43-S44)</f>
-        <v>-114439.93922766112</v>
+        <v>-113594.23106224654</v>
       </c>
       <c r="U45" s="13">
         <f>-a_tax*MAX(0,U43-T44)</f>
-        <v>-116109.18954958877</v>
+        <v>-115246.56722086592</v>
       </c>
       <c r="V45" s="13">
         <f>-a_tax*MAX(0,V43-U44)</f>
-        <v>-117811.82487795502</v>
+        <v>-116931.9501026577</v>
       </c>
       <c r="W45" s="13">
         <f>-a_tax*MAX(0,W43-V44)</f>
-        <v>-122216.57658819955</v>
+        <v>-121319.10431739625</v>
       </c>
     </row>
     <row r="46" spans="1:23">
@@ -26052,87 +26052,87 @@
       </c>
       <c r="C48" s="14">
         <f>C20+C45+C21*(1-a_debt_frac)+C22+C23+C25-C38-C39+C41+C42</f>
-        <v>-2127118.484630888</v>
+        <v>-2126961.8781148875</v>
       </c>
       <c r="D48" s="14">
         <f>D20+D45+D21*(1-a_debt_frac)+D22+D23+D25-D38-D39+D41+D42</f>
-        <v>-111315.14757592784</v>
+        <v>-113855.11691240556</v>
       </c>
       <c r="E48" s="14">
         <f>E20+E45+E21*(1-a_debt_frac)+E22+E23+E25-E38-E39+E41+E42</f>
-        <v>675341.8274683922</v>
+        <v>672487.1382317224</v>
       </c>
       <c r="F48" s="14">
         <f>F20+F45+F21*(1-a_debt_frac)+F22+F23+F25-F38-F39+F41+F42</f>
-        <v>305491.07727116207</v>
+        <v>302612.52434721834</v>
       </c>
       <c r="G48" s="14">
         <f>G20+G45+G21*(1-a_debt_frac)+G22+G23+G25-G38-G39+G41+G42</f>
-        <v>316321.4672044565</v>
+        <v>313384.74081199314</v>
       </c>
       <c r="H48" s="14">
         <f>H20+H45+H21*(1-a_debt_frac)+H22+H23+H25-H38-H39+H41+H42</f>
-        <v>321892.2374912757</v>
+        <v>318896.1741609225</v>
       </c>
       <c r="I48" s="14">
         <f>I20+I45+I21*(1-a_debt_frac)+I22+I23+I25-I38-I39+I41+I42</f>
-        <v>327574.4231838313</v>
+        <v>324517.8361768305</v>
       </c>
       <c r="J48" s="14">
         <f>J20+J45+J21*(1-a_debt_frac)+J22+J23+J25-J38-J39+J41+J42</f>
-        <v>333370.252590238</v>
+        <v>330251.93143305636</v>
       </c>
       <c r="K48" s="14">
         <f>K20+K45+K21*(1-a_debt_frac)+K22+K23+K25-K38-K39+K41+K42</f>
-        <v>124165.33623275673</v>
+        <v>120984.04624239105</v>
       </c>
       <c r="L48" s="14">
         <f>L20+L45+L21*(1-a_debt_frac)+L22+L23+L25-L38-L39+L41+L42</f>
-        <v>345311.9794991984</v>
+        <v>342066.4612989847</v>
       </c>
       <c r="M48" s="14">
         <f>M20+M45+M21*(1-a_debt_frac)+M22+M23+M25-M38-M39+M41+M42</f>
-        <v>508133.6831356805</v>
+        <v>511443.1878023844</v>
       </c>
       <c r="N48" s="14">
         <f>N20+N45+N21*(1-a_debt_frac)+N22+N23+N25-N38-N39+N41+N42</f>
-        <v>509132.32410820236</v>
+        <v>506475.3142509574</v>
       </c>
       <c r="O48" s="14">
         <f>O20+O45+O21*(1-a_debt_frac)+O22+O23+O25-O38-O39+O41+O42</f>
-        <v>338327.3083439745</v>
+        <v>335617.1582895847</v>
       </c>
       <c r="P48" s="14">
         <f>P20+P45+P21*(1-a_debt_frac)+P22+P23+P25-P38-P39+P41+P42</f>
-        <v>424027.62518986035</v>
+        <v>421263.27213438274</v>
       </c>
       <c r="Q48" s="14">
         <f>Q20+Q45+Q21*(1-a_debt_frac)+Q22+Q23+Q25-Q38-Q39+Q41+Q42</f>
-        <v>429459.2466350722</v>
+        <v>426639.606518485</v>
       </c>
       <c r="R48" s="14">
         <f>R20+R45+R21*(1-a_debt_frac)+R22+R23+R25-R38-R39+R41+R42</f>
-        <v>434999.5005091883</v>
+        <v>432123.46759026934</v>
       </c>
       <c r="S48" s="14">
         <f>S20+S45+S21*(1-a_debt_frac)+S22+S23+S25-S38-S39+S41+S42</f>
-        <v>189622.59081647222</v>
+        <v>186689.03723917488</v>
       </c>
       <c r="T48" s="14">
         <f>T20+T45+T21*(1-a_debt_frac)+T22+T23+T25-T38-T39+T41+T42</f>
-        <v>447430.126401739</v>
+        <v>444437.90175289573</v>
       </c>
       <c r="U48" s="14">
         <f>U20+U45+U21*(1-a_debt_frac)+U22+U23+U25-U38-U39+U41+U42</f>
-        <v>453309.4881349819</v>
+        <v>450257.4189931619</v>
       </c>
       <c r="V48" s="14">
         <f>V20+V45+V21*(1-a_debt_frac)+V22+V23+V25-V38-V39+V41+V42</f>
-        <v>459306.43710288976</v>
+        <v>456193.32657823333</v>
       </c>
       <c r="W48" s="14">
         <f>W20+W45+W21*(1-a_debt_frac)+W22+W23+W25-W38-W39+W41+W42</f>
-        <v>598311.9423162618</v>
+        <v>594801.2748348593</v>
       </c>
     </row>
     <row r="50" spans="1:1">
@@ -26181,7 +26181,7 @@
       </c>
       <c r="B4" s="3">
         <f>SUMPRODUCT('Arus Kas'!$C$31:$W$31,'Arus Kas'!$C$33:$W$33)</f>
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>372</v>
@@ -26197,7 +26197,7 @@
       </c>
       <c r="B5" s="4">
         <f>IRR('Arus Kas'!$C$31:$W$31)</f>
-        <v>0.12225595720238847</v>
+        <v>0.12150604052544578</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>374</v>
@@ -26213,7 +26213,7 @@
       </c>
       <c r="B6" s="4">
         <f>IRR('Arus Kas'!$C$48:$W$48)</f>
-        <v>0.14128956808421878</v>
+        <v>0.14006099840090447</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>376</v>
@@ -26245,7 +26245,7 @@
       </c>
       <c r="B8" s="5">
         <f>SUM('Arus Kas'!$C$36:$W$36)</f>
-        <v>6.345177407024556</v>
+        <v>6.369787840205327</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>378</v>
@@ -26261,7 +26261,7 @@
       </c>
       <c r="B9" s="5">
         <f>IF(SUM('Arus Kas'!$C$37:$W$37)=0,"&gt; umur",SUM('Arus Kas'!$C$37:$W$37))</f>
-        <v>12.294909064732625</v>
+        <v>12.431932646836765</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>378</v>
@@ -26277,7 +26277,7 @@
       </c>
       <c r="B10" s="5">
         <f>SUMPRODUCT('Arus Kas'!$D$31:$W$31,'Arus Kas'!$D$33:$W$33)/FCI</f>
-        <v>1.2822753549647496</v>
+        <v>1.2768608143095233</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>381</v>
@@ -26293,7 +26293,7 @@
       </c>
       <c r="B11" s="5">
         <f>MIN('Arus Kas'!$C$47:$W$47)</f>
-        <v>1.3180782341273873</v>
+        <v>1.3056039524321026</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>383</v>
@@ -26309,7 +26309,7 @@
       </c>
       <c r="B12" s="11">
         <f>(FCI-SUMPRODUCT('Arus Kas'!$C$18:$W$18,'Arus Kas'!$C$33:$W$33)-SUMPRODUCT('Arus Kas'!$C$19:$W$19,'Arus Kas'!$C$33:$W$33)-SUMPRODUCT('Arus Kas'!$C$22:$W$22,'Arus Kas'!$C$33:$W$33))/(SUMPRODUCT('Arus Kas'!$C$7:$W$7,'Arus Kas'!$C$33:$W$33)*1000000)</f>
-        <v>0.18495651125562335</v>
+        <v>0.18562485764138928</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>385</v>
@@ -26325,7 +26325,7 @@
       </c>
       <c r="B13" s="3">
         <f>-MIN('Arus Kas'!$C$32:$W$32)</f>
-        <v>4546175.134666292</v>
+        <v>4545840.428041292</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>387</v>
@@ -26361,7 +26361,7 @@
         <v>390</v>
       </c>
       <c r="B17" s="10">
-        <v>0.5828638963044959</v>
+        <v>0.5961118395426859</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -26369,7 +26369,7 @@
         <v>391</v>
       </c>
       <c r="B18" s="10">
-        <v>2.775542363354742</v>
+        <v>2.838627807346124</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -26377,7 +26377,7 @@
         <v>392</v>
       </c>
       <c r="B19" s="10">
-        <v>5.888993638139839</v>
+        <v>6.02527292016077</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -26385,7 +26385,7 @@
         <v>393</v>
       </c>
       <c r="B20" s="10">
-        <v>-1.953261772455062</v>
+        <v>-1.732431169527921</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -26393,7 +26393,7 @@
         <v>394</v>
       </c>
       <c r="B21" s="10">
-        <v>0.5825751882375558</v>
+        <v>0.5936708599962552</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -26401,7 +26401,7 @@
         <v>395</v>
       </c>
       <c r="B22" s="10">
-        <v>1.164554184286368</v>
+        <v>1.159338532513162</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -26417,7 +26417,7 @@
         <v>397</v>
       </c>
       <c r="B24" s="15">
-        <v>0.5905637741275449</v>
+        <v>0.5947845781888141</v>
       </c>
     </row>
   </sheetData>
@@ -26462,17 +26462,17 @@
         <v>404</v>
       </c>
       <c r="B4" s="13">
-        <v>-543041.0958787735</v>
+        <v>-565947.8995100182</v>
       </c>
       <c r="C4" s="13">
-        <v>1898771.815638745</v>
+        <v>1877400.087390472</v>
       </c>
       <c r="D4" s="12">
         <f>ABS(C4-B4)</f>
-        <v>2441812.911517518</v>
+        <v>2443347.98690049</v>
       </c>
       <c r="E4" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -26480,17 +26480,17 @@
         <v>405</v>
       </c>
       <c r="B5" s="13">
-        <v>1522618.336499129</v>
+        <v>1501194.317101539</v>
       </c>
       <c r="C5" s="13">
-        <v>-153781.6032148016</v>
+        <v>-176398.1055447065</v>
       </c>
       <c r="D5" s="12">
         <f>ABS(C5-B5)</f>
-        <v>1676399.9397139305</v>
+        <v>1677592.4226462457</v>
       </c>
       <c r="E5" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -26498,17 +26498,17 @@
         <v>406</v>
       </c>
       <c r="B6" s="13">
-        <v>95385.42794068452</v>
+        <v>72939.60458279701</v>
       </c>
       <c r="C6" s="13">
-        <v>1303226.533249845</v>
+        <v>1281578.000547802</v>
       </c>
       <c r="D6" s="12">
         <f>ABS(C6-B6)</f>
-        <v>1207841.1053091602</v>
+        <v>1208638.3959650053</v>
       </c>
       <c r="E6" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -26516,17 +26516,17 @@
         <v>407</v>
       </c>
       <c r="B7" s="13">
-        <v>1217388.51427597</v>
+        <v>1200115.990392726</v>
       </c>
       <c r="C7" s="13">
-        <v>184385.4201327429</v>
+        <v>157396.6066132198</v>
       </c>
       <c r="D7" s="12">
         <f>ABS(C7-B7)</f>
-        <v>1033003.0941432267</v>
+        <v>1042719.3837795061</v>
       </c>
       <c r="E7" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -26534,17 +26534,17 @@
         <v>408</v>
       </c>
       <c r="B8" s="13">
-        <v>303643.8459021507</v>
+        <v>281198.0225442628</v>
       </c>
       <c r="C8" s="13">
-        <v>1098989.672646724</v>
+        <v>1077165.61516268</v>
       </c>
       <c r="D8" s="12">
         <f>ABS(C8-B8)</f>
-        <v>795345.826744573</v>
+        <v>795967.5926184176</v>
       </c>
       <c r="E8" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -26552,17 +26552,17 @@
         <v>409</v>
       </c>
       <c r="B9" s="13">
-        <v>1115586.89586406</v>
+        <v>1091340.884232128</v>
       </c>
       <c r="C9" s="13">
-        <v>342909.2159653</v>
+        <v>322438.9103750603</v>
       </c>
       <c r="D9" s="12">
         <f>ABS(C9-B9)</f>
-        <v>772677.6798987602</v>
+        <v>768901.9738570675</v>
       </c>
       <c r="E9" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -26570,17 +26570,17 @@
         <v>410</v>
       </c>
       <c r="B10" s="13">
-        <v>367897.2974386065</v>
+        <v>345451.474080719</v>
       </c>
       <c r="C10" s="13">
-        <v>1038629.338581595</v>
+        <v>1016611.371747759</v>
       </c>
       <c r="D10" s="12">
         <f>ABS(C10-B10)</f>
-        <v>670732.0411429888</v>
+        <v>671159.8976670397</v>
       </c>
       <c r="E10" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -26588,17 +26588,17 @@
         <v>411</v>
       </c>
       <c r="B11" s="13">
-        <v>404807.6603446143</v>
+        <v>382361.8369867256</v>
       </c>
       <c r="C11" s="13">
-        <v>935810.8738326941</v>
+        <v>913910.6180240845</v>
       </c>
       <c r="D11" s="12">
         <f>ABS(C11-B11)</f>
-        <v>531003.2134880798</v>
+        <v>531548.7810373589</v>
       </c>
       <c r="E11" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -26606,17 +26606,17 @@
         <v>412</v>
       </c>
       <c r="B12" s="13">
-        <v>605528.068883601</v>
+        <v>583082.2455257138</v>
       </c>
       <c r="C12" s="13">
-        <v>804802.5829811528</v>
+        <v>782784.6161473172</v>
       </c>
       <c r="D12" s="12">
         <f>ABS(C12-B12)</f>
-        <v>199274.51409755182</v>
+        <v>199702.37062160345</v>
       </c>
       <c r="E12" s="12">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -26638,7 +26638,7 @@
       </c>
       <c r="B17" s="13">
         <f>'Arus Kas'!$C$31+NPV(A17,'Arus Kas'!$D$31:$W$31)</f>
-        <v>3269267.1996731823</v>
+        <v>3233928.145940558</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -26647,7 +26647,7 @@
       </c>
       <c r="B18" s="13">
         <f>'Arus Kas'!$C$31+NPV(A18,'Arus Kas'!$D$31:$W$31)</f>
-        <v>2972567.0333865928</v>
+        <v>2938797.2024187334</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -26656,7 +26656,7 @@
       </c>
       <c r="B19" s="13">
         <f>'Arus Kas'!$C$31+NPV(A19,'Arus Kas'!$D$31:$W$31)</f>
-        <v>2693302.568581547</v>
+        <v>2660999.066889058</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -26665,7 +26665,7 @@
       </c>
       <c r="B20" s="13">
         <f>'Arus Kas'!$C$31+NPV(A20,'Arus Kas'!$D$31:$W$31)</f>
-        <v>2430195.517452772</v>
+        <v>2399263.4820770836</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -26674,7 +26674,7 @@
       </c>
       <c r="B21" s="13">
         <f>'Arus Kas'!$C$31+NPV(A21,'Arus Kas'!$D$31:$W$31)</f>
-        <v>2182074.8672046014</v>
+        <v>2152426.7692785813</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -26683,7 +26683,7 @@
       </c>
       <c r="B22" s="13">
         <f>'Arus Kas'!$C$31+NPV(A22,'Arus Kas'!$D$31:$W$31)</f>
-        <v>1947866.9894888161</v>
+        <v>1919422.003034134</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -26692,7 +26692,7 @@
       </c>
       <c r="B23" s="13">
         <f>'Arus Kas'!$C$31+NPV(A23,'Arus Kas'!$D$31:$W$31)</f>
-        <v>1726586.7297566542</v>
+        <v>1699270.159213186</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -26701,7 +26701,7 @@
       </c>
       <c r="B24" s="13">
         <f>'Arus Kas'!$C$31+NPV(A24,'Arus Kas'!$D$31:$W$31)</f>
-        <v>1517329.3735594128</v>
+        <v>1491072.1342262463</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -26710,7 +26710,7 @@
       </c>
       <c r="B25" s="13">
         <f>'Arus Kas'!$C$31+NPV(A25,'Arus Kas'!$D$31:$W$31)</f>
-        <v>1319263.3982093295</v>
+        <v>1294001.5443856898</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -26719,7 +26719,7 @@
       </c>
       <c r="B26" s="13">
         <f>'Arus Kas'!$C$31+NPV(A26,'Arus Kas'!$D$31:$W$31)</f>
-        <v>1131623.9282763898</v>
+        <v>1107298.2244328542</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -26728,7 +26728,7 @@
       </c>
       <c r="B27" s="13">
         <f>'Arus Kas'!$C$31+NPV(A27,'Arus Kas'!$D$31:$W$31)</f>
-        <v>953706.8223032231</v>
+        <v>930262.3530964057</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -26737,7 +26737,7 @@
       </c>
       <c r="B28" s="13">
         <f>'Arus Kas'!$C$31+NPV(A28,'Arus Kas'!$D$31:$W$31)</f>
-        <v>784863.3260097193</v>
+        <v>762249.1413840966</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -26746,7 +26746,7 @@
       </c>
       <c r="B29" s="13">
         <f>'Arus Kas'!$C$31+NPV(A29,'Arus Kas'!$D$31:$W$31)</f>
-        <v>624495.2342506241</v>
+        <v>602664.0262551631</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -26755,7 +26755,7 @@
       </c>
       <c r="B30" s="13">
         <f>'Arus Kas'!$C$31+NPV(A30,'Arus Kas'!$D$31:$W$31)</f>
-        <v>472050.51019139664</v>
+        <v>450958.3184813967</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -26764,7 +26764,7 @@
       </c>
       <c r="B31" s="13">
         <f>'Arus Kas'!$C$31+NPV(A31,'Arus Kas'!$D$31:$W$31)</f>
-        <v>327019.3156711395</v>
+        <v>306625.2589719249</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -26773,7 +26773,7 @@
       </c>
       <c r="B32" s="13">
         <f>'Arus Kas'!$C$31+NPV(A32,'Arus Kas'!$D$31:$W$31)</f>
-        <v>188930.41161014634</v>
+        <v>169196.4426928563</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -26782,7 +26782,7 @@
       </c>
       <c r="B33" s="13">
         <f>'Arus Kas'!$C$31+NPV(A33,'Arus Kas'!$D$31:$W$31)</f>
-        <v>57347.89166374598</v>
+        <v>38238.573628280894</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -26791,7 +26791,7 @@
       </c>
       <c r="B34" s="13">
         <f>'Arus Kas'!$C$31+NPV(A34,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-68131.78381224057</v>
+        <v>-86649.4819330393</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -26800,7 +26800,7 @@
       </c>
       <c r="B35" s="13">
         <f>'Arus Kas'!$C$31+NPV(A35,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-187882.48298077402</v>
+        <v>-205839.37308546156</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -26809,7 +26809,7 @@
       </c>
       <c r="B36" s="13">
         <f>'Arus Kas'!$C$31+NPV(A36,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-302250.8533621847</v>
+        <v>-319675.6992275151</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -26818,7 +26818,7 @@
       </c>
       <c r="B37" s="13">
         <f>'Arus Kas'!$C$31+NPV(A37,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-411558.55199828476</v>
+        <v>-428478.2257648624</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -26827,7 +26827,7 @@
       </c>
       <c r="B38" s="13">
         <f>'Arus Kas'!$C$31+NPV(A38,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-516104.27621552773</v>
+        <v>-532543.9017272156</v>
       </c>
     </row>
     <row r="39" spans="1:2">
@@ -26836,7 +26836,7 @@
       </c>
       <c r="B39" s="13">
         <f>'Arus Kas'!$C$31+NPV(A39,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-616165.6140897981</v>
+        <v>-632148.6982749056</v>
       </c>
     </row>
     <row r="40" spans="1:2">
@@ -26845,7 +26845,7 @@
       </c>
       <c r="B40" s="13">
         <f>'Arus Kas'!$C$31+NPV(A40,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-712000.7317777171</v>
+        <v>-727549.2851458985</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -26854,7 +26854,7 @@
       </c>
       <c r="B41" s="13">
         <f>'Arus Kas'!$C$31+NPV(A41,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-803849.9131475608</v>
+        <v>-818984.560373871</v>
       </c>
     </row>
     <row r="42" spans="1:2">
@@ -26863,7 +26863,7 @@
       </c>
       <c r="B42" s="13">
         <f>'Arus Kas'!$C$31+NPV(A42,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-891936.965595297</v>
+        <v>-906677.0470706664</v>
       </c>
     </row>
     <row r="43" spans="1:2">
@@ -26872,7 +26872,7 @@
       </c>
       <c r="B43" s="13">
         <f>'Arus Kas'!$C$31+NPV(A43,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-976470.5045463681</v>
+        <v>-990834.1696907661</v>
       </c>
     </row>
     <row r="44" spans="1:2">
@@ -26881,7 +26881,7 @@
       </c>
       <c r="B44" s="13">
         <f>'Arus Kas'!$C$31+NPV(A44,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1057645.1279046785</v>
+        <v>-1071649.4209645549</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -26890,7 +26890,7 @@
       </c>
       <c r="B45" s="13">
         <f>'Arus Kas'!$C$31+NPV(A45,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1135642.490599939</v>
+        <v>-1149303.4295841798</v>
       </c>
     </row>
     <row r="46" spans="1:2">
@@ -26899,7 +26899,7 @@
       </c>
       <c r="B46" s="13">
         <f>'Arus Kas'!$C$31+NPV(A46,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1210632.2883898343</v>
+        <v>-1223964.9377378388</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -26908,7 +26908,7 @@
       </c>
       <c r="B47" s="13">
         <f>'Arus Kas'!$C$31+NPV(A47,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1282773.1591811022</v>
+        <v>-1295791.6967017895</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -26917,7 +26917,7 @@
       </c>
       <c r="B48" s="13">
         <f>'Arus Kas'!$C$31+NPV(A48,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1352213.509333176</v>
+        <v>-1364931.2879043529</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -26926,7 +26926,7 @@
       </c>
       <c r="B49" s="13">
         <f>'Arus Kas'!$C$31+NPV(A49,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1419092.271689017</v>
+        <v>-1431521.8761619083</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -26935,7 +26935,7 @@
       </c>
       <c r="B50" s="13">
         <f>'Arus Kas'!$C$31+NPV(A50,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1483539.6014320944</v>
+        <v>-1495692.9011455283</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -26944,7 +26944,7 @@
       </c>
       <c r="B51" s="13">
         <f>'Arus Kas'!$C$31+NPV(A51,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1545677.515287707</v>
+        <v>-1557565.7125599594</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -26953,7 +26953,7 @@
       </c>
       <c r="B52" s="13">
         <f>'Arus Kas'!$C$31+NPV(A52,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1605620.4790647118</v>
+        <v>-1617254.153998071</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -26962,7 +26962,7 @@
       </c>
       <c r="B53" s="13">
         <f>'Arus Kas'!$C$31+NPV(A53,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1663475.948063523</v>
+        <v>-1674865.0999667633</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -26971,7 +26971,7 @@
       </c>
       <c r="B54" s="13">
         <f>'Arus Kas'!$C$31+NPV(A54,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1719344.864452985</v>
+        <v>-1730498.950159903</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -26980,7 +26980,7 @@
       </c>
       <c r="B55" s="13">
         <f>'Arus Kas'!$C$31+NPV(A55,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1773322.1153371783</v>
+        <v>-1784250.0846748513</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -26989,7 +26989,7 @@
       </c>
       <c r="B56" s="13">
         <f>'Arus Kas'!$C$31+NPV(A56,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1825496.9548892095</v>
+        <v>-1836207.2835274225</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -26998,7 +26998,7 @@
       </c>
       <c r="B57" s="13">
         <f>'Arus Kas'!$C$31+NPV(A57,'Arus Kas'!$D$31:$W$31)</f>
-        <v>-1875953.39361871</v>
+        <v>-1886454.113511846</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -27028,16 +27028,16 @@
         <v>422</v>
       </c>
       <c r="B62" s="12">
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
       <c r="C62" s="13">
-        <v>705580.1216725706</v>
+        <v>683353.7257154244</v>
       </c>
       <c r="D62" s="15">
-        <v>0.1222559572023885</v>
+        <v>0.1215060405254458</v>
       </c>
       <c r="E62" s="10">
-        <v>6.345177407024556</v>
+        <v>6.369787840205327</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -27045,16 +27045,16 @@
         <v>423</v>
       </c>
       <c r="B63" s="12">
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
       <c r="C63" s="13">
-        <v>-1006874.759175735</v>
+        <v>-1030255.933197843</v>
       </c>
       <c r="D63" s="15">
-        <v>0.0571692469201821</v>
+        <v>0.05614013402345552</v>
       </c>
       <c r="E63" s="10">
-        <v>9.472204013077191</v>
+        <v>9.528146815493713</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -27062,16 +27062,16 @@
         <v>424</v>
       </c>
       <c r="B64" s="12">
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
       <c r="C64" s="13">
-        <v>-781824.2484732983</v>
+        <v>-804731.0521045423</v>
       </c>
       <c r="D64" s="15">
-        <v>0.06387322919803462</v>
+        <v>0.06279156195873759</v>
       </c>
       <c r="E64" s="10">
-        <v>8.514441923307368</v>
+        <v>8.560344473124211</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -27079,16 +27079,16 @@
         <v>425</v>
       </c>
       <c r="B65" s="12">
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
       <c r="C65" s="13">
-        <v>1030575.327328429</v>
+        <v>1008751.269844385</v>
       </c>
       <c r="D65" s="15">
-        <v>0.1336435645263003</v>
+        <v>0.1329265577238703</v>
       </c>
       <c r="E65" s="10">
-        <v>5.90910356576318</v>
+        <v>5.925801569681511</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -27096,16 +27096,16 @@
         <v>426</v>
       </c>
       <c r="B66" s="12">
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
       <c r="C66" s="13">
-        <v>731607.0209493645</v>
+        <v>709397.5614115016</v>
       </c>
       <c r="D66" s="15">
-        <v>0.1218531847341813</v>
+        <v>0.1211351310631499</v>
       </c>
       <c r="E66" s="10">
-        <v>6.345177407024556</v>
+        <v>6.369787840205327</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -27113,16 +27113,16 @@
         <v>427</v>
       </c>
       <c r="B67" s="12">
-        <v>3369956.060270474</v>
+        <v>3369707.951346837</v>
       </c>
       <c r="C67" s="13">
-        <v>1431447.786953798</v>
+        <v>1410029.732101631</v>
       </c>
       <c r="D67" s="15">
-        <v>0.1559750738192469</v>
+        <v>0.1551880106746895</v>
       </c>
       <c r="E67" s="10">
-        <v>5.394369610457598</v>
+        <v>5.411022097985593</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -27130,16 +27130,16 @@
         <v>428</v>
       </c>
       <c r="B68" s="12">
-        <v>3091100.094171512</v>
+        <v>3090798.556671512</v>
       </c>
       <c r="C68" s="13">
-        <v>-261376.6039165471</v>
+        <v>-280988.9768581073</v>
       </c>
       <c r="D68" s="15">
-        <v>0.08467361028058584</v>
+        <v>0.08368893017776169</v>
       </c>
       <c r="E68" s="10">
-        <v>8.266776315316202</v>
+        <v>8.314460568672715</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -27147,16 +27147,16 @@
         <v>429</v>
       </c>
       <c r="B69" s="12">
-        <v>5051182.956913788</v>
+        <v>5050881.419413787</v>
       </c>
       <c r="C69" s="13">
-        <v>1604787.385872489</v>
+        <v>1580216.797938611</v>
       </c>
       <c r="D69" s="15">
-        <v>0.1420065157462997</v>
+        <v>0.14137553093577</v>
       </c>
       <c r="E69" s="10">
-        <v>5.749928463165156</v>
+        <v>5.764513003338198</v>
       </c>
     </row>
   </sheetData>
@@ -27199,13 +27199,13 @@
         <v>432</v>
       </c>
       <c r="B4" s="13">
-        <v>-815692.854356139</v>
+        <v>-837584.6983127948</v>
       </c>
       <c r="C4" s="15">
-        <v>0.07261884807428824</v>
+        <v>0.07172135552377382</v>
       </c>
       <c r="D4" s="10">
-        <v>5.935070127006009</v>
+        <v>5.955046741831567</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -27213,13 +27213,13 @@
         <v>433</v>
       </c>
       <c r="B5" s="13">
-        <v>187647.4737772103</v>
+        <v>164092.3251144696</v>
       </c>
       <c r="C5" s="15">
-        <v>0.1044449764831934</v>
+        <v>0.1037074871113444</v>
       </c>
       <c r="D5" s="10">
-        <v>7.108837649536074</v>
+        <v>7.150908379399169</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -27227,13 +27227,13 @@
         <v>434</v>
       </c>
       <c r="B6" s="13">
-        <v>1115753.866508945</v>
+        <v>1094904.2683524</v>
       </c>
       <c r="C6" s="15">
-        <v>0.1355799517377584</v>
+        <v>0.134850222400026</v>
       </c>
       <c r="D6" s="10">
-        <v>9.101965511683584</v>
+        <v>9.14916286626463</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -27241,7 +27241,7 @@
         <v>435</v>
       </c>
       <c r="B7" s="13">
-        <v>172074.6199153156</v>
+        <v>148258.9199845902</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -27249,7 +27249,7 @@
         <v>436</v>
       </c>
       <c r="B9" s="4">
-        <v>0.609</v>
+        <v>0.5943333333333334</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -27257,7 +27257,7 @@
         <v>437</v>
       </c>
       <c r="B10" s="4">
-        <v>0.6156666666666667</v>
+        <v>0.5996666666666667</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -27293,7 +27293,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="10">
-        <v>0.6744700464966717</v>
+        <v>0.6743407864823096</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>443</v>
@@ -27304,7 +27304,7 @@
         <v>444</v>
       </c>
       <c r="B16" s="10">
-        <v>-0.5562957666995295</v>
+        <v>-0.5560084786676086</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>445</v>
@@ -27315,7 +27315,7 @@
         <v>446</v>
       </c>
       <c r="B17" s="10">
-        <v>0.2356258030695337</v>
+        <v>0.2356437959604217</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>447</v>
@@ -27326,7 +27326,7 @@
         <v>448</v>
       </c>
       <c r="B18" s="10">
-        <v>-0.2101515446835049</v>
+        <v>-0.2120359537817726</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>449</v>
@@ -27337,7 +27337,7 @@
         <v>50</v>
       </c>
       <c r="B19" s="10">
-        <v>0.132753154305906</v>
+        <v>0.1327439551937728</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>450</v>
@@ -27348,7 +27348,7 @@
         <v>451</v>
       </c>
       <c r="B20" s="10">
-        <v>0.1251740716860079</v>
+        <v>0.1251497263499696</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>452</v>
@@ -27359,7 +27359,7 @@
         <v>141</v>
       </c>
       <c r="B21" s="10">
-        <v>-0.1176712019634669</v>
+        <v>-0.1167741005304556</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>453</v>
@@ -27370,7 +27370,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="10">
-        <v>0.08028648669849853</v>
+        <v>0.08029185025465001</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>454</v>
@@ -27381,7 +27381,7 @@
         <v>40</v>
       </c>
       <c r="B23" s="10">
-        <v>0.07543826349314038</v>
+        <v>0.07543298882588764</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>455</v>
@@ -27392,7 +27392,7 @@
         <v>456</v>
       </c>
       <c r="B24" s="10">
-        <v>-0.07502449589161064</v>
+        <v>-0.07505966656218516</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>457</v>
@@ -27403,7 +27403,7 @@
         <v>73</v>
       </c>
       <c r="B25" s="10">
-        <v>0.05580073153341461</v>
+        <v>0.05464679540519948</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>458</v>
@@ -27414,7 +27414,7 @@
         <v>18</v>
       </c>
       <c r="B26" s="10">
-        <v>0.04414442846049205</v>
+        <v>0.04419634179959352</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>459</v>
@@ -27425,7 +27425,7 @@
         <v>54</v>
       </c>
       <c r="B27" s="10">
-        <v>0.0236251959583551</v>
+        <v>0.0235622035069115</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>460</v>
@@ -27441,23 +27441,23 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="12">
-        <v>-2206213.721122548</v>
+        <v>-2232479.874163236</v>
       </c>
       <c r="B31" s="12">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="12">
-        <v>-2041185.286519913</v>
+        <v>-2067363.791636461</v>
       </c>
       <c r="B32" s="12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="12">
-        <v>-1876156.85191728</v>
+        <v>-1902247.709109687</v>
       </c>
       <c r="B33" s="12">
         <v>5</v>
@@ -27465,7 +27465,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="12">
-        <v>-1711128.417314646</v>
+        <v>-1737131.626582914</v>
       </c>
       <c r="B34" s="12">
         <v>10</v>
@@ -27473,7 +27473,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="12">
-        <v>-1546099.982712012</v>
+        <v>-1572015.54405614</v>
       </c>
       <c r="B35" s="12">
         <v>27</v>
@@ -27481,71 +27481,71 @@
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="12">
-        <v>-1381071.548109378</v>
+        <v>-1406899.461529366</v>
       </c>
       <c r="B36" s="12">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="12">
-        <v>-1216043.113506744</v>
+        <v>-1241783.379002592</v>
       </c>
       <c r="B37" s="12">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="12">
-        <v>-1051014.67890411</v>
+        <v>-1076667.296475818</v>
       </c>
       <c r="B38" s="12">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="12">
-        <v>-885986.2443014761</v>
+        <v>-911551.2139490441</v>
       </c>
       <c r="B39" s="12">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="12">
-        <v>-720957.8096988421</v>
+        <v>-746435.1314222702</v>
       </c>
       <c r="B40" s="12">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="12">
-        <v>-555929.3750962083</v>
+        <v>-581319.0488954963</v>
       </c>
       <c r="B41" s="12">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="12">
-        <v>-390900.9404935744</v>
+        <v>-416202.9663687225</v>
       </c>
       <c r="B42" s="12">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="12">
-        <v>-225872.5058909403</v>
+        <v>-251086.8838419486</v>
       </c>
       <c r="B43" s="12">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="12">
-        <v>-60844.0712883065</v>
+        <v>-85970.80131517467</v>
       </c>
       <c r="B44" s="12">
         <v>236</v>
@@ -27553,7 +27553,7 @@
     </row>
     <row r="45" spans="1:2">
       <c r="A45" s="12">
-        <v>104184.3633143273</v>
+        <v>79145.28121159924</v>
       </c>
       <c r="B45" s="12">
         <v>283</v>
@@ -27561,63 +27561,63 @@
     </row>
     <row r="46" spans="1:2">
       <c r="A46" s="12">
-        <v>269212.7979169614</v>
+        <v>244261.3637383732</v>
       </c>
       <c r="B46" s="12">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="12">
-        <v>434241.2325195954</v>
+        <v>409377.4462651468</v>
       </c>
       <c r="B47" s="12">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="12">
-        <v>599269.6671222295</v>
+        <v>574493.5287919207</v>
       </c>
       <c r="B48" s="12">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="12">
-        <v>764298.1017248633</v>
+        <v>739609.6113186947</v>
       </c>
       <c r="B49" s="12">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50" s="12">
-        <v>929326.5363274971</v>
+        <v>904725.6938454686</v>
       </c>
       <c r="B50" s="12">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" s="12">
-        <v>1094354.970930131</v>
+        <v>1069841.776372242</v>
       </c>
       <c r="B51" s="12">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" s="12">
-        <v>1259383.405532765</v>
+        <v>1234957.858899016</v>
       </c>
       <c r="B52" s="12">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" s="12">
-        <v>1424411.840135399</v>
+        <v>1400073.94142579</v>
       </c>
       <c r="B53" s="12">
         <v>67</v>
@@ -27625,23 +27625,23 @@
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="12">
-        <v>1589440.274738033</v>
+        <v>1565190.023952564</v>
       </c>
       <c r="B54" s="12">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="12">
-        <v>1754468.709340667</v>
+        <v>1730306.106479338</v>
       </c>
       <c r="B55" s="12">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="12">
-        <v>1919497.143943301</v>
+        <v>1895422.189006112</v>
       </c>
       <c r="B56" s="12">
         <v>10</v>
@@ -27649,7 +27649,7 @@
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="12">
-        <v>2084525.578545935</v>
+        <v>2060538.271532886</v>
       </c>
       <c r="B57" s="12">
         <v>4</v>
@@ -27657,7 +27657,7 @@
     </row>
     <row r="58" spans="1:2">
       <c r="A58" s="12">
-        <v>2249554.013148569</v>
+        <v>2225654.354059659</v>
       </c>
       <c r="B58" s="12">
         <v>0</v>
@@ -27665,7 +27665,7 @@
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="12">
-        <v>2414582.447751202</v>
+        <v>2390770.436586434</v>
       </c>
       <c r="B59" s="12">
         <v>3</v>
@@ -27673,7 +27673,7 @@
     </row>
     <row r="60" spans="1:2">
       <c r="A60" s="12">
-        <v>2579610.882353836</v>
+        <v>2555886.519113207</v>
       </c>
       <c r="B60" s="12">
         <v>1</v>
@@ -27732,13 +27732,13 @@
         <v>418</v>
       </c>
       <c r="B5" s="12">
-        <v>3091100.094171512</v>
+        <v>3090798.556671512</v>
       </c>
       <c r="C5" s="12">
-        <v>4095653.274474137</v>
+        <v>4095351.736974137</v>
       </c>
       <c r="D5" s="12">
-        <v>5051182.956913788</v>
+        <v>5050881.419413787</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -27774,13 +27774,13 @@
         <v>419</v>
       </c>
       <c r="B8" s="13">
-        <v>-261376.6039165471</v>
+        <v>-280988.9768581073</v>
       </c>
       <c r="C8" s="13">
-        <v>633326.2475301967</v>
+        <v>611099.8515730508</v>
       </c>
       <c r="D8" s="13">
-        <v>1604787.385872489</v>
+        <v>1580216.797938611</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -27788,13 +27788,13 @@
         <v>420</v>
       </c>
       <c r="B9" s="15">
-        <v>0.08467361028058584</v>
+        <v>0.08368893017776169</v>
       </c>
       <c r="C9" s="15">
-        <v>0.1197406094098632</v>
+        <v>0.1189868519171766</v>
       </c>
       <c r="D9" s="15">
-        <v>0.1420065157462997</v>
+        <v>0.14137553093577</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -27802,13 +27802,13 @@
         <v>421</v>
       </c>
       <c r="B10" s="10">
-        <v>8.266776315316202</v>
+        <v>8.314460568672715</v>
       </c>
       <c r="C10" s="10">
-        <v>6.444124334563693</v>
+        <v>6.469579125492325</v>
       </c>
       <c r="D10" s="10">
-        <v>5.749928463165156</v>
+        <v>5.764513003338198</v>
       </c>
     </row>
     <row r="12" spans="1:4">

</xml_diff>